<commit_message>
Address LOT2-5 spec review: CAR-T provenance, disenrollment split, AUTO trigger, dynamic flags
- Reword CAR-T 45-day window as Apr 22 study-team decision (resolved Q11),
  not 'per protocol'.
- Split LOT end logic into PRIMARY (ignores disenrollment) and SENSITIVITY
  (CENSOR_AT_DISENROLLMENT=TRUE caps via ENDDATE_CE and emits DISENROLLMENT
  reason). Adds LOTN_BASE_END_DT_CE_SENS / LOTN_BASE_END_REASON_CE_SENS
  rows and a new sensitivity scenario S6b. Resolved Q12.
- Promote unplanned AUTO to a first-class competing LOT-start trigger in
  LOTN_START_DT and SCT_CART_LOT_START sheets.
- Add dynamic LOTN_MED_[MED] and LOTN_CLASS_[CLASS] flag rows mirroring
  LOT1 output.
- Clarify maintenance follows current LOT1 CODE behaviour (not protocol
  Rule 8 wording) on cover and Q5.
- Make builder path repo-relative via Path(__file__) so it works on any
  checkout; default CHUNK=all so a fresh run produces the full workbook.
- Fix NOC -> NDC, 'Inducton' -> 'Induction'.
</commit_message>
<xml_diff>
--- a/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
+++ b/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -745,7 +745,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Inherits LOT1 approach: contains_mtx_reg flag, no standalone maintenance LOT</t>
+          <t>Follows current LOT1 CODE behaviour (descriptive contains_mtx_reg flag; no standalone maintenance LOT). Diverges from the protocol Rule 8 wording. Open Q5.</t>
         </is>
       </c>
     </row>
@@ -770,6 +770,30 @@
       <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Excluded from regimen identification (per LOT1 protocol Section 5.1.1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>CAR-T consolidation</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>45 days (per Apr 22 study-team decision; supersedes 30-day older protocol text). Resolved Q11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Disenrollment</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>PRIMARY analysis: ignored. SENSITIVITY (CENSOR_AT_DISENROLLMENT=TRUE) caps via ENDDATE_CE and emits DISENROLLMENT reason. Resolved Q12.</t>
         </is>
       </c>
     </row>
@@ -897,7 +921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1013,7 +1037,7 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Earliest of: (a) first MM oncology agent (non-steroid) administered/dispensed AFTER LOT_(N-1)_BASE_END_DT; (b) first ALLO SCT date AFTER LOT_(N-1)_BASE_END_DT (ALLO always starts a new LOT); (c) first CAR-T infusion date AFTER LOT_(N-1)_BASE_END_DT (CAR-T classified as its own LOT). If LOT_(N-1) ended due to SCT_ALLO/SCT_CART/CART_INIT/SCT_AUTO unplanned, LOTN_START_DT = the SCT/CAR-T event date itself.</t>
+          <t>LOTN_START_DT is the EARLIEST of any of the following competing triggers occurring after LOT_(N-1)_BASE_END_DT: (a) first MM oncology agent (non-steroid) administered/dispensed; (b) first autologous SCT (AUTO) - including an unplanned AUTO (&gt;180 days after a prior AUTO in LOT_(N-1)); (c) first allogeneic SCT (ALLO) - ALLO always starts a new LOT; (d) first CAR-T infusion - CAR-T is classified as its own LOT. When LOT_(N-1) ended due to SCT_ALLO / SCT_CART / SCT_AUTO unplanned / CART_INIT, LOTN_START_DT equals the SCT or CAR-T event date itself (LOT_(N-1) ended the day before that event).</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -1023,7 +1047,7 @@
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>Source: T_MEDICAL (PROC_CD, BILL_PROC_CD, NOC), T_RX (NOC), T_MEDICAL procedure codes for SCT/CAR-T. Steroids excluded from medication-trigger candidates (MAP_MED_CLASS != 'STEROID'). Permissible biosimilar subs do NOT trigger a new LOT.</t>
+          <t>Source: T_MEDICAL (PROC_CD, BILL_PROC_CD, NDC), T_RX (NDC), T_MEDICAL procedure codes for SCT/CAR-T. Steroids excluded from medication-trigger candidates (MAP_MED_CLASS != 'STEROID'). Permissible biosimilar substitutions do NOT trigger a new LOT.</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr"/>
@@ -1051,7 +1075,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Indicates which trigger started LOT N: a new MM medication, an autologous SCT (unplanned), an allogeneic SCT, or a CAR-T infusion.</t>
+          <t>Indicates which trigger started LOT N: a new MM medication, an unplanned autologous SCT, an allogeneic SCT, or a CAR-T infusion. All four are first-class competing triggers - whichever is earliest defines LOTN_START_DT and LOTN_START_TYPE.</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -1188,32 +1212,32 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>LOTN_TX_AUTO_FLG</t>
+          <t>LOTN_MED_[MED]</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Flag: any valid AUTO SCT during LOT N</t>
+          <t>Per-medication induction flags (one column per MED_ABBR)</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>0 / 1</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Binary flag indicating the patient received any valid autologous SCT during LOT N (single or tandem).</t>
+          <t>For each distinct medication abbreviation in CL_MMA_ROLLUP (Tab 40), emit a flag column LOTN_MED_BORT, LOTN_MED_LENA, LOTN_MED_DARA, LOTN_MED_CARF, LOTN_MED_IXAZ, LOTN_MED_THAL, LOTN_MED_POMA, LOTN_MED_CYCL, LOTN_MED_MELP, LOTN_MED_BEND, LOTN_MED_IDEC, LOTN_MED_CILT, LOTN_MED_BELA, LOTN_MED_ISAT, LOTN_MED_ELOT, LOTN_MED_ETOP, LOTN_MED_PANO, LOTN_MED_SELI, LOTN_MED_TECL, LOTN_MED_DOPL, LOTN_MED_DOXO, LOTN_MED_CISP, LOTN_MED_ELRA, LOTN_MED_LINV, LOTN_MED_TALQ, LOTN_MED_VENE, etc. = 1 if that medication is part of LOTN_BASE_MEDS.</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>CL_SCT_CODELIST (SCT_TYPE='AUTO')</t>
+          <t>CL_MMA_ROLLUP (Tab 40), CL_MMA_CODELIST (Tab 41)</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Same logic as LOT1: 14-day windowing of T_MEDICAL procedure code dates; 60-day gap validation between distinct events.</t>
+          <t>Mirror LOT1 dynamic flag generation. Steroid abbreviations (DEXA, PRED) excluded since regimen excludes steroids.</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr"/>
@@ -1226,32 +1250,32 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>LOTN_TX_AUTO_SING_FL</t>
+          <t>LOTN_CLASS_[CLASS]</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Flag: single valid AUTO SCT during LOT N</t>
+          <t>Per-class induction flags (one column per MED_CLASS)</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>0 / 1</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Single AUTO not part of a valid tandem pair within LOT N.</t>
+          <t>For each MED_CLASS in CL_MMA_ROLLUP, emit a flag column: LOTN_CLASS_PROTINHIB, LOTN_CLASS_IMMUNOMOD, LOTN_CLASS_ANTICD38, LOTN_CLASS_BCMA, LOTN_CLASS_MUSTARD, LOTN_CLASS_SIGNALING, LOTN_CLASS_TOPOISOMERASE, LOTN_CLASS_HDACINHIBITOR, LOTN_CLASS_XPORTINHIBITOR, LOTN_CLASS_ANTHRACYCLINE, LOTN_CLASS_PLATINUM, LOTN_CLASS_CELMOD, LOTN_CLASS_BCL2INHIBITOR. = 1 if any agent of that class is in LOTN_BASE_MEDS.</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>CL_SCT_CODELIST</t>
+          <t>CL_MMA_ROLLUP MED_CLASS</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Inherits LOT1 SCT logic.</t>
+          <t>Mirror LOT1 dynamic class flag generation. STEROID class excluded.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr"/>
@@ -1264,12 +1288,12 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>LOTN_TX_AUTO_TAND_FL</t>
+          <t>LOTN_TX_AUTO_FLG</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Flag: planned tandem AUTO SCT during LOT N</t>
+          <t>Flag: any valid AUTO SCT during LOT N</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -1279,17 +1303,17 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Two AUTO SCTs within LOT N that are &gt;=60 and &lt;=180 days apart (planned tandem).</t>
+          <t>Binary flag indicating the patient received any valid autologous SCT during LOT N (single or tandem).</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>CL_SCT_CODELIST</t>
+          <t>CL_SCT_CODELIST (SCT_TYPE='AUTO')</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Use datediff(AUTO_DT_2, AUTO_DT_1) without +1 (per Apr 22 protocol resolution).</t>
+          <t>Same logic as LOT1: 14-day windowing of T_MEDICAL procedure code dates; 60-day gap validation between distinct events.</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr"/>
@@ -1302,22 +1326,22 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>LOTN_TX_AUTO_DT_1 / LOTN_TX_AUTO_DT_2</t>
+          <t>LOTN_TX_AUTO_SING_FL</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Dates of first/second valid AUTO during LOT N</t>
+          <t>Flag: single valid AUTO SCT during LOT N</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Date / Date</t>
+          <t>0/1</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>AUTO_DT_1 is the first valid AUTO SCT during LOT N; AUTO_DT_2 is the second when a planned tandem exists.</t>
+          <t>Single AUTO not part of a valid tandem pair within LOT N.</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -1327,7 +1351,7 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>14-day windowing groups same-event claims; 60-day gap validates distinct events.</t>
+          <t>Inherits LOT1 SCT logic.</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr"/>
@@ -1340,22 +1364,22 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>LOTN_TX_AUTO_MAX_DT</t>
+          <t>LOTN_TX_AUTO_TAND_FL</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Latest valid AUTO SCT date during LOT N</t>
+          <t>Flag: planned tandem AUTO SCT during LOT N</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>0/1</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Date of AUTO_DT_2 if a valid tandem; else AUTO_DT_1 if a single AUTO occurred; else NULL.</t>
+          <t>Two AUTO SCTs within LOT N that are &gt;=60 and &lt;=180 days apart (planned tandem).</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -1363,7 +1387,11 @@
           <t>CL_SCT_CODELIST</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr"/>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Use datediff(AUTO_DT_2, AUTO_DT_1) without +1 (per Apr 22 protocol resolution).</t>
+        </is>
+      </c>
       <c r="H12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
@@ -1374,32 +1402,32 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>contains_mtx_reg_LOTN</t>
+          <t>LOTN_TX_AUTO_DT_1 / LOTN_TX_AUTO_DT_2</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Flag: LOT N regimen contains valid maintenance subset</t>
+          <t>Dates of first/second valid AUTO during LOT N</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>0 / 1</t>
+          <t>Date / Date</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Set 1 when LOT N induction regimen contains BOTH (a) at least one valid mono-maintenance agent OR a valid dual-maintenance combination, AND (b) at least one additional non-maintenance anchor agent. Same definition as LOT1. Valid mono: lenalidomide, bortezomib, daratumumab, ixazomib, thalidomide. Valid dual: bortezomib/lenalidomide, carfilzomib/lenalidomide, daratumumab/lenalidomide.</t>
+          <t>AUTO_DT_1 is the first valid AUTO SCT during LOT N; AUTO_DT_2 is the second when a planned tandem exists.</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>CL_MMA_ROLLUP MONOMAINTENANCE / DUALMAINTENANCEWITH</t>
+          <t>CL_SCT_CODELIST</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Descriptive flag only; does NOT derive a separate maintenance LOT or maintenance end date.</t>
+          <t>14-day windowing groups same-event claims; 60-day gap validates distinct events.</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr"/>
@@ -1412,34 +1440,30 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>LOTN_ALLO_LOT_FLG</t>
+          <t>LOTN_TX_AUTO_MAX_DT</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Flag: LOT N is an allogeneic SCT line</t>
+          <t>Latest valid AUTO SCT date during LOT N</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Set 1 when LOTN_START_TYPE='SCT_ALLO'. Per protocol: an allogeneic SCT is classified as its own LOT, with no other MM therapies included in that LOT. LOT span is the ALLO date itself (start = end = ALLO date) unless followed by a regimen that initiates LOT_(N+1).</t>
+          <t>Date of AUTO_DT_2 if a valid tandem; else AUTO_DT_1 if a single AUTO occurred; else NULL.</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>CL_SCT_CODELIST (SCT_TYPE='ALLO')</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>Open question: should LOTN_BASE_END_DT be the ALLO date (one-day LOT) or extend to the day before LOT_(N+1) start? See Open_Questions tab Q2.</t>
-        </is>
-      </c>
+          <t>CL_SCT_CODELIST</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr"/>
       <c r="H14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
@@ -1450,35 +1474,111 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
+          <t>contains_mtx_reg_LOTN</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Flag: LOT N regimen contains valid maintenance subset</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>0 / 1</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Set 1 when LOT N induction regimen contains BOTH (a) at least one valid mono-maintenance agent OR a valid dual-maintenance combination, AND (b) at least one additional non-maintenance anchor agent. Same definition as LOT1. Valid mono: lenalidomide, bortezomib, daratumumab, ixazomib, thalidomide. Valid dual: bortezomib/lenalidomide, carfilzomib/lenalidomide, daratumumab/lenalidomide.</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>CL_MMA_ROLLUP MONOMAINTENANCE / DUALMAINTENANCEWITH</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Descriptive flag only; does NOT derive a separate maintenance LOT or maintenance end date.</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>FU_PD</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>LOTN_ALLO_LOT_FLG</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Flag: LOT N is an allogeneic SCT line</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Set 1 when LOTN_START_TYPE='SCT_ALLO'. Per protocol: an allogeneic SCT is classified as its own LOT, with no other MM therapies included in that LOT. LOT span is the ALLO date itself (start = end = ALLO date) unless followed by a regimen that initiates LOT_(N+1).</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>CL_SCT_CODELIST (SCT_TYPE='ALLO')</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Open question: should LOTN_BASE_END_DT be the ALLO date (one-day LOT) or extend to the day before LOT_(N+1) start? See Open_Questions tab Q2.</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>FU_PD</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
           <t>LOTN_CART_LOT_FLG</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>Flag: LOT N is a CAR-T line</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>0/1</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>Set 1 when LOTN_START_TYPE='CART'. Per protocol: CAR-T is its own LOT; oncology agents (incl. supportive, e.g., corticosteroids) given within 45 days of CAR-T are CONSOLIDATED into the CAR-T LOT and not treated as new induction.</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>CL_SCT_CODELIST (SCT_TYPE='CART')</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>Within 45-day consolidation window, do NOT advance to LOT_(N+1). Use FIRST_CART_DT as LOTN_START_DT.</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr"/>
+      <c r="H17" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1491,7 +1591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1569,17 +1669,17 @@
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>LOT N continues until the earliest of: (1) Discontinuation of all agents in the regimen (with or without switch to a new agent) - end date is the run-out date (last MAP_END_DT among induction agents); (2) Addition of a qualifying new MM oncology agent not in the LOT N induction regimen and not a permissible biosimilar substitute - end date is the day before the new agent's MAP_START_DT; (3) SCT/CAR-T events: any ALLO SCT ends the LOT the day before the ALLO; an AUTO SCT &gt;180 days after a previous AUTO ends LOT the day before; CAR-T infusion ends the LOT the day before FIRST_CART_DT; (4) Death; (5) Health plan disenrollment; (6) End of the study period.</t>
+          <t>PRIMARY analysis - LOT N continues until the earliest of: (1) Discontinuation of all agents in the regimen (with or without switch to a new agent) - end date is the run-out date (last MAP_END_DT among induction agents); (2) Addition of a qualifying new MM oncology agent not in the LOT N induction regimen and not a permissible biosimilar substitute - end date is the day before the new agent's MAP_START_DT; (3) SCT/CAR-T events: any ALLO SCT ends the LOT the day before the ALLO; an AUTO SCT &gt;180 days after a previous AUTO ends LOT the day before; CAR-T infusion ends the LOT the day before FIRST_CART_DT; (4) Death (T_DOD.YMDOD); (5) End of the study period (study_end config). Health plan disenrollment is NOT a primary LOT-ending event. SENSITIVITY analysis - when CENSOR_AT_DISENROLLMENT = TRUE, LOT N observation end is additionally capped at ENDDATE_CE (see LOTN_END_REASON_CE_SENS below).</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>T_MEDICAL/T_RX (MAP_END_DT, MAP_START_DT), T_MEDICAL procedure codes (SCT/CAR-T), T_DOD (YMDOD), T_MEMBER_CONT_ENROLLMENT (ELIGEND), study_end config</t>
+          <t>T_MEDICAL/T_RX (MAP_END_DT, MAP_START_DT), T_MEDICAL procedure codes (SCT/CAR-T), T_DOD (YMDOD), study_end config; SENSITIVITY only: T_MEMBER_CONT_ENROLLMENT (ELIGEND -&gt; ENDDATE_CE)</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
-          <t>Same priority logic as LOT1; only the induction window differs.</t>
+          <t>Primary path mirrors current LOT1 implementation: ignores disenrollment. Same priority logic as LOT1; only the induction window differs.</t>
         </is>
       </c>
       <c r="H2" s="7" t="inlineStr"/>
@@ -1820,22 +1920,22 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>CART_45D_CONSOLIDATION</t>
+          <t>CART_CONSOLIDATION_DAYS</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>CAR-T 45-day consolidation rule</t>
+          <t>CAR-T consolidation window (days)</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>45</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Oncology therapies (including supportive agents like steroids) given within 45 days of FIRST_CART_DT are consolidated into the CAR-T LOT.</t>
+          <t>Oncology therapies (including supportive agents like steroids) given within 45 days of FIRST_CART_DT are consolidated into the CAR-T LOT. PROVENANCE: per Apr 22, 2026 study-team decision, the CAR-T consolidation window is 45 days. This supersedes the earlier 30-day language in the protocol extract; treat 45 as the operative value for LOT2-5 (matches LOT1 CART_INIT).</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -1845,7 +1945,7 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Reclassify within 45-day window; do NOT trigger LOT_(N+1).</t>
+          <t>Reclassify therapies within 45-day window into the CAR-T LOT; do NOT trigger LOT_(N+1) for those agents.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr"/>
@@ -1901,22 +2001,22 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Final LOT N base end reason</t>
+          <t>Final LOT N base end reason (PRIMARY analysis)</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>SCT_ALLO / SCT_CART / SCT_AUTO / CART_INIT / MED_ADD / DISCONTINUATION / DEATH / DISENROLLMENT / STUDY_END</t>
+          <t>SCT_ALLO / SCT_CART / SCT_AUTO / CART_INIT / MED_ADD / DISCONTINUATION / DEATH / STUDY_END</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Final reason. Priority when ties on the same day: SCT_ALLO &gt; SCT_CART &gt; SCT_AUTO &gt; CART_INIT &gt; MED_ADD &gt; DISCONTINUATION &gt; DEATH &gt; DISENROLLMENT &gt; STUDY_END.</t>
+          <t>Final reason for the PRIMARY analysis. Priority when ties on the same day: SCT_ALLO &gt; SCT_CART &gt; SCT_AUTO &gt; CART_INIT &gt; MED_ADD &gt; DISCONTINUATION &gt; DEATH &gt; STUDY_END. DISENROLLMENT is NOT a primary end reason - it appears only in the sensitivity output (LOTN_BASE_END_REASON_CE_SENS).</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>All sources above</t>
+          <t>All sources above (excluding T_MEMBER_CONT_ENROLLMENT for primary)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1934,32 +2034,32 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>LOTN_BASE_LENGTH</t>
+          <t>LOTN_BASE_END_DT_CE_SENS</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>LOT N base period duration in days</t>
+          <t>LOT N base end date - sensitivity (censor at disenrollment)</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Integer</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>If LOTN_BASE_END_REASON = 'DISCONTINUATION' then LOTN_BASE_DISCON_DT - LOTN_START_DT + 1; else LOTN_BASE_END_DT - LOTN_START_DT + 1.</t>
+          <t>Sensitivity-analysis end date computed identically to LOTN_BASE_END_DT but additionally capped at ENDDATE_CE = min(YMDOD, ELIGEND, study_end). Only emitted when CENSOR_AT_DISENROLLMENT = TRUE.</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>T_MEMBER_CONT_ENROLLMENT (ELIGEND), T_DOD, study_end config</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Confirm censored-patient handling against LOT1 M1 finding (Apr 15 review).</t>
+          <t>Sensitivity flag-gated; primary LOTN_BASE_END_DT remains untouched.</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr"/>
@@ -1972,35 +2072,111 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
+          <t>LOTN_BASE_END_REASON_CE_SENS</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>LOT N base end reason - sensitivity</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>SCT_ALLO / SCT_CART / SCT_AUTO / CART_INIT / MED_ADD / DISCONTINUATION / DEATH / DISENROLLMENT / STUDY_END</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Final reason for the sensitivity analysis. DISENROLLMENT is emitted when ELIGEND is the binding earliest cap. Priority order extends the primary list: SCT_ALLO &gt; SCT_CART &gt; SCT_AUTO &gt; CART_INIT &gt; MED_ADD &gt; DISCONTINUATION &gt; DEATH &gt; DISENROLLMENT &gt; STUDY_END.</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>All sources above plus T_MEMBER_CONT_ENROLLMENT (ELIGEND)</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>REQUIRED behaviour: when sensitivity ENDDATE_CE binds because of disenrollment (ELIGEND earliest), label the reason DISENROLLMENT (do NOT collapse to STUDY_END). This is a deliberate divergence from the current LOT1 implementation, which labels the cap as STUDY_END; LOT2-5 should emit DISENROLLMENT for analytic clarity.</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>FU_PD</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_LENGTH</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>LOT N base period duration in days</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>If LOTN_BASE_END_REASON = 'DISCONTINUATION' then LOTN_BASE_DISCON_DT - LOTN_START_DT + 1; else LOTN_BASE_END_DT - LOTN_START_DT + 1.</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Confirm censored-patient handling against LOT1 M1 finding (Apr 15 review).</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>FU_PD</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
           <t>PERMISSIBLE_SUBS_EFFECT</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Permissible biosimilar substitution rules</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>Do not advance LOT</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT. The LOT is named by the drug given for the longest duration.</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>permissible_subs reference</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>Same as LOT1.</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr"/>
+      <c r="H15" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2106,7 +2282,7 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>Includes all oncology therapies (and supportive agents like steroids) within 45 days post-CAR-T (consolidation).</t>
+          <t>Includes all oncology therapies (and supportive agents like steroids) within 45 days post-CAR-T (consolidation per Apr 22 decision).</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -2116,7 +2292,7 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Use 45-day consolidation window for the CAR-T LOT regimen.</t>
+          <t>Use 45-day consolidation window per Apr 22 study-team decision (supersedes 30-day protocol text).</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2304,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>AUTO occurs &gt;180 days after a previous AUTO in the same line.</t>
+          <t>AUTO occurs &gt;180 days after a previous AUTO in the same line. Competes as a first-class LOT-start trigger alongside MED, ALLO, CAR-T - whichever is earliest wins.</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -2138,7 +2314,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Inducton window 30 days from AUTO_DT.</t>
+          <t>Induction window 30 days from AUTO_DT.</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -2227,7 +2403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2357,66 +2533,83 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>S7. Tandem AUTO during LOT2</t>
+          <t>S6b. Disenrollment during LOT3 (primary vs sensitivity)</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Two AUTO SCTs 90 days apart during LOT2.</t>
+          <t>Patient disenrolls (ELIGEND) during LOT3 with no death and no further therapy. Study end is later.</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Both are planned tandem; LOT2 continues. LOT2_TX_AUTO_TAND_FL = 1; LOT2_TX_AUTO_DT_1/DT_2 populated. LOT2 does not end on the second AUTO.</t>
+          <t>PRIMARY: disenrollment is ignored. LOT3_BASE_END_REASON = STUDY_END (earliest of death/study_end), LOT3_BASE_END_DT = study_end. SENSITIVITY (CENSOR_AT_DISENROLLMENT=TRUE): LOT3_BASE_END_DT_CE_SENS = ELIGEND; LOT3_BASE_END_REASON_CE_SENS = DISENROLLMENT.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>S8. Permissible biosimilar swap mid-LOT2</t>
+          <t>S7. Tandem AUTO during LOT2</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Patient on DARA in LOT2 switches to a DARA biosimilar.</t>
+          <t>Two AUTO SCTs 90 days apart during LOT2.</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Substitution does NOT advance the LOT. LOT2 continues; regimen named by drug with longest duration.</t>
+          <t>Both are planned tandem; LOT2 continues. LOT2_TX_AUTO_TAND_FL = 1; LOT2_TX_AUTO_DT_1/DT_2 populated. LOT2 does not end on the second AUTO.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>S9. LOT2 base length = 1 day (ALLO LOT, open question)</t>
+          <t>S8. Permissible biosimilar swap mid-LOT2</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>ALLO is its own LOT; if no further therapy, what is LOT span?</t>
+          <t>Patient on DARA in LOT2 switches to a DARA biosimilar.</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Open question Q2. Draft assumption: LOT2_BASE_END_DT = ALLO_DT (1-day LOT); subsequent agents -&gt; LOT3.</t>
+          <t>Substitution does NOT advance the LOT. LOT2 continues; regimen named by drug with longest duration.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
+          <t>S9. LOT2 base length = 1 day (ALLO LOT, open question)</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>ALLO is its own LOT; if no further therapy, what is LOT span?</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Open question Q2. Draft assumption: LOT2_BASE_END_DT = ALLO_DT (1-day LOT); subsequent agents -&gt; LOT3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
           <t>S10. CART_INIT carries through LOT boundary</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>First add medication appears in LOT1, CAR-T occurs within 45 days of that add.</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Per LOT1 spec: LOT1_BASE_END_REASON = CART_INIT and LOT1_BASE_END_DT = FIRST_CART_DT - 1. LOT2_START_TYPE = CART; FIRST_CART_DT = LOT2_START_DT.</t>
         </is>
@@ -2433,7 +2626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2591,7 +2784,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Draft: NO - matches LOT1 decision (no standalone maintenance LOT). Use contains_mtx_reg_LOTN flag only.</t>
+          <t>Draft: NO - follows current LOT1 CODE behaviour (no standalone maintenance LOT) rather than the protocol Rule 8 wording. Use contains_mtx_reg_LOTN flag only. If the team later reverses this for LOT1, LOT2-5 should follow.</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -2737,6 +2930,60 @@
       <c r="E11" s="7" t="inlineStr">
         <is>
           <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>CAR-T consolidation window: 45 vs 30 days.</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>RESOLVED: 45 days. Per Apr 22 study-team decision; supersedes the 30-day language in the older protocol extract. Document as Apr 22 decision in spec, NOT 'per protocol'.</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Julia</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Disenrollment as a LOT end event: primary vs sensitivity treatment.</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>RESOLVED: PRIMARY analysis ignores disenrollment - LOT N ends only on regimen events, SCT/CAR-T events, death, or study_end. SENSITIVITY analysis (CENSOR_AT_DISENROLLMENT=TRUE) caps observation at ENDDATE_CE = min(YMDOD, ELIGEND, study_end) and emits DISENROLLMENT as the end reason when ELIGEND binds. Spec requires the implementation to label sensitivity reason DISENROLLMENT (not collapse to STUDY_END as current LOT1 code does).</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Julia</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Resolved</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tighten LOT2-5 spec wording: unplanned-AUTO trigger, CAR-T provenance, sensitivity-only disenrollment
- LOTN_START_DT: trigger is the first UNPLANNED autologous SCT; planned/
  single/tandem AUTO are continuations and do NOT start a new LOT.
- LOTN_CART_LOT_FLG: drop 'Per protocol' phrasing; cite Apr 22 study-team
  decision for the 45-day consolidation window.
- SCT_CART_LOT_START sheet: split the death/disenrollment/study-end row
  into PRIMARY (death + study end) and SENSITIVITY-ONLY (disenrollment via
  ENDDATE_CE) so a reader using that sheet alone can't infer disenrollment
  ends follow-up under the primary analysis.
</commit_message>
<xml_diff>
--- a/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
+++ b/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
@@ -1037,7 +1037,7 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>LOTN_START_DT is the EARLIEST of any of the following competing triggers occurring after LOT_(N-1)_BASE_END_DT: (a) first MM oncology agent (non-steroid) administered/dispensed; (b) first autologous SCT (AUTO) - including an unplanned AUTO (&gt;180 days after a prior AUTO in LOT_(N-1)); (c) first allogeneic SCT (ALLO) - ALLO always starts a new LOT; (d) first CAR-T infusion - CAR-T is classified as its own LOT. When LOT_(N-1) ended due to SCT_ALLO / SCT_CART / SCT_AUTO unplanned / CART_INIT, LOTN_START_DT equals the SCT or CAR-T event date itself (LOT_(N-1) ended the day before that event).</t>
+          <t>LOTN_START_DT is the EARLIEST of any of the following competing triggers occurring after LOT_(N-1)_BASE_END_DT: (a) first MM oncology agent (non-steroid) administered/dispensed; (b) first UNPLANNED autologous SCT (AUTO) - i.e., an AUTO occurring &gt;180 days after a prior AUTO in LOT_(N-1). Planned, single, or tandem AUTO SCTs (60-180 day intervals) are continuations of the same LOT and do NOT trigger a new LOT; (c) first allogeneic SCT (ALLO) - ALLO always starts a new LOT; (d) first CAR-T infusion - CAR-T is classified as its own LOT. When LOT_(N-1) ended due to SCT_ALLO / SCT_CART / SCT_AUTO unplanned / CART_INIT, LOTN_START_DT equals the SCT or CAR-T event date itself (LOT_(N-1) ended the day before that event).</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Set 1 when LOTN_START_TYPE='CART'. Per protocol: CAR-T is its own LOT; oncology agents (incl. supportive, e.g., corticosteroids) given within 45 days of CAR-T are CONSOLIDATED into the CAR-T LOT and not treated as new induction.</t>
+          <t>Set 1 when LOTN_START_TYPE='CART'. CAR-T is its own LOT; oncology agents (incl. supportive, e.g., corticosteroids) given within 45 days of CAR-T are CONSOLIDATED into the CAR-T LOT and not treated as new induction. PROVENANCE: 45-day consolidation per Apr 22 study-team decision (supersedes 30-day older protocol text); see Q11.</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
@@ -2189,7 +2189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2363,7 +2363,7 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Death / disenrollment / study end</t>
+          <t>Death / study end (PRIMARY)</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -2383,12 +2383,44 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>DEATH / DISENROLLMENT / STUDY_END</t>
+          <t>DEATH / STUDY_END</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>LOT_(N-1) ends; no new LOT begins.</t>
+          <t>LOT_(N-1) ends; no new LOT begins. Disenrollment is NOT a primary end event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Health plan disenrollment (SENSITIVITY ONLY)</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Never starts a new LOT. Sensitivity-only: when CENSOR_AT_DISENROLLMENT=TRUE, ELIGEND caps observation via ENDDATE_CE.</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>DISENROLLMENT (sensitivity only; primary analysis ignores ELIGEND)</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>PRIMARY analysis does NOT use disenrollment to end any LOT. SENSITIVITY emits LOTN_BASE_END_DT_CE_SENS / LOTN_BASE_END_REASON_CE_SENS only when the sensitivity flag is on. See Q12.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LOT2-5 spec: standardize AUTO flag suffix to _FLG; clean docstring
- Rename LOTN_TX_AUTO_SING_FL/TAND_FL -> LOTN_TX_AUTO_SING_FLG/TAND_FLG
  to match LOT1 naming convention. Also updated the scenario reference
  that used the old suffix.
- Drop the unsupported 'finalize' value from the CHUNK docstring; list
  the actual chunks (cover, qc, base, base_end, sct_cart, scenarios,
  open_q, all) and note 'all' is the default.
</commit_message>
<xml_diff>
--- a/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
+++ b/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
@@ -1326,7 +1326,7 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>LOTN_TX_AUTO_SING_FL</t>
+          <t>LOTN_TX_AUTO_SING_FLG</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>LOTN_TX_AUTO_TAND_FL</t>
+          <t>LOTN_TX_AUTO_TAND_FLG</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Both are planned tandem; LOT2 continues. LOT2_TX_AUTO_TAND_FL = 1; LOT2_TX_AUTO_DT_1/DT_2 populated. LOT2 does not end on the second AUTO.</t>
+          <t>Both are planned tandem; LOT2 continues. LOT2_TX_AUTO_TAND_FLG = 1; LOT2_TX_AUTO_DT_1/DT_2 populated. LOT2 does not end on the second AUTO.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LOT2-5 spec: add worked examples, Gantt timelines, and decision-flow sheet
- Append worked-example appendices to LOT2_5_BASE (Examples A/B/C: med-
  triggered LOT2, ALLO-started LOT2, unplanned-AUTO-started LOT2) and
  LOT2_5_BASE_END (Examples D/E/F: end-reason priority with CART_INIT,
  discontinuation, disenrollment primary vs sensitivity).
- New sheet 8.Timelines: Gantt-style patient journeys for 7 scenarios,
  with a colored legend, day axis (14-day buckets), LOT segments,
  induction-window overlays, and event markers (M/A/X/C/+).
- New sheet 9.Decision_Flow: 6-step decision tree for when LOT(N+1)
  starts, with same-day tie-break priority noted.
- Cover updated with the two new tabs.
</commit_message>
<xml_diff>
--- a/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
+++ b/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
@@ -14,6 +14,8 @@
     <sheet name="5.SCT_CART_LOT_START" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="6.Scenarios" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="7.Open_Questions" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="8.Timelines" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="9.Decision_Flow" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,8 +54,49 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -70,8 +113,78 @@
         <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0070AD47"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4B084"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6E0B4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B4A7D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF9900"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007030A0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00404040"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000070C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -93,11 +206,69 @@
         <color rgb="00999999"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top style="medium">
+        <color rgb="00FFE699"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -116,6 +287,90 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -483,7 +738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -690,108 +945,132 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr"/>
-      <c r="B20" s="3" t="inlineStr"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>8.Timelines</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Gantt-style patient journey examples (visual)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>9.Decision_Flow</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Decision tree for when LOT(N+1) starts</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Key differences vs LOT1</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Induction window</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>30 days (vs 60 days for LOT1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>LOT start trigger</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>First MM oncology agent OR ALLO SCT OR CAR-T event (vs LOT1 = first MM agent only)</t>
-        </is>
-      </c>
+      <c r="B23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Numbering</t>
+          <t>Induction window</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>LOT_NUM increments 2..5; same algorithmic rules otherwise</t>
+          <t>30 days (vs 60 days for LOT1)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>LOT start trigger</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Follows current LOT1 CODE behaviour (descriptive contains_mtx_reg flag; no standalone maintenance LOT). Diverges from the protocol Rule 8 wording. Open Q5.</t>
+          <t>First MM oncology agent OR ALLO SCT OR CAR-T event (vs LOT1 = first MM agent only)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Permissible subs</t>
+          <t>Numbering</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Same as LOT1 - do not advance LOT</t>
+          <t>LOT_NUM increments 2..5; same algorithmic rules otherwise</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Steroids</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Excluded from regimen identification (per LOT1 protocol Section 5.1.1)</t>
+          <t>Follows current LOT1 CODE behaviour (descriptive contains_mtx_reg flag; no standalone maintenance LOT). Diverges from the protocol Rule 8 wording. Open Q5.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>CAR-T consolidation</t>
+          <t>Permissible subs</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>45 days (per Apr 22 study-team decision; supersedes 30-day older protocol text). Resolved Q11.</t>
+          <t>Same as LOT1 - do not advance LOT</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t>Steroids</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Excluded from regimen identification (per LOT1 protocol Section 5.1.1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>CAR-T consolidation</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>45 days (per Apr 22 study-team decision; supersedes 30-day older protocol text). Resolved Q11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
           <t>Disenrollment</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>PRIMARY analysis: ignored. SENSITIVITY (CENSOR_AT_DISENROLLMENT=TRUE) caps via ENDDATE_CE and emits DISENROLLMENT reason. Resolved Q12.</t>
         </is>
@@ -921,7 +1200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1580,7 +1859,751 @@
       </c>
       <c r="H17" s="7" t="inlineStr"/>
     </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>WORKED EXAMPLE A - LOT2 starts on a new medication</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Example A - LOT2 starts on a NEW MEDICATION (most common case).
+Patient was on VRd (bortezomib + lenalidomide + dexamethasone) for LOT1. LOT1 ended on 2025-08-19 with reason MED_ADD because daratumumab was added on 2025-08-20. The patient receives DARA on 2025-08-20 and lenalidomide refills appear within 30 days. No SCT or CAR-T occurs.</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="n"/>
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="10" t="n"/>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="10" t="n"/>
+      <c r="H21" s="11" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Value for this patient</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>How it was derived</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="n"/>
+      <c r="E22" s="12" t="n"/>
+      <c r="F22" s="12" t="n"/>
+      <c r="G22" s="12" t="n"/>
+      <c r="H22" s="12" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>LOT_NUM</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Sequential index after LOT1.</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="9" t="n"/>
+      <c r="F23" s="9" t="n"/>
+      <c r="G23" s="9" t="n"/>
+      <c r="H23" s="9" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_START_DT</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>2025-08-20</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Earliest competing trigger after LOT1_BASE_END_DT (2025-08-19) is the new MM agent DARA on 2025-08-20.</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="n"/>
+      <c r="E24" s="9" t="n"/>
+      <c r="F24" s="9" t="n"/>
+      <c r="G24" s="9" t="n"/>
+      <c r="H24" s="9" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_START_TYPE</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Trigger was a new medication (no SCT/CAR-T present).</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="9" t="n"/>
+      <c r="F25" s="9" t="n"/>
+      <c r="G25" s="9" t="n"/>
+      <c r="H25" s="9" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>INDUCTION_WINDOW_DAYS</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>LOT2 uses the 30-day induction window (vs 60 for LOT1).</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="9" t="n"/>
+      <c r="F26" s="9" t="n"/>
+      <c r="G26" s="9" t="n"/>
+      <c r="H26" s="9" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_MEDS</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>DARA, LENA</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Within [2025-08-20, 2025-09-18]: DARA (start) and LENA refills. DEXA excluded (steroid).</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="n"/>
+      <c r="E27" s="9" t="n"/>
+      <c r="F27" s="9" t="n"/>
+      <c r="G27" s="9" t="n"/>
+      <c r="H27" s="9" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_MED_CNT</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Two distinct non-steroid agents.</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="n"/>
+      <c r="E28" s="9" t="n"/>
+      <c r="F28" s="9" t="n"/>
+      <c r="G28" s="9" t="n"/>
+      <c r="H28" s="9" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_MED_DARA</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>DARA present in LOTN_BASE_MEDS.</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="9" t="n"/>
+      <c r="F29" s="9" t="n"/>
+      <c r="G29" s="9" t="n"/>
+      <c r="H29" s="9" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_MED_LENA</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>LENA present in LOTN_BASE_MEDS.</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="n"/>
+      <c r="E30" s="9" t="n"/>
+      <c r="F30" s="9" t="n"/>
+      <c r="G30" s="9" t="n"/>
+      <c r="H30" s="9" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_CLASS_ANTICD38</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>DARA is class ANTICD38.</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="n"/>
+      <c r="E31" s="9" t="n"/>
+      <c r="F31" s="9" t="n"/>
+      <c r="G31" s="9" t="n"/>
+      <c r="H31" s="9" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_CLASS_IMMUNOMOD</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>LENA is class IMMUNOMOD.</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="n"/>
+      <c r="E32" s="9" t="n"/>
+      <c r="F32" s="9" t="n"/>
+      <c r="G32" s="9" t="n"/>
+      <c r="H32" s="9" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>contains_mtx_reg_LOTN</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>LENA is a valid mono-maintenance agent (a); DARA is the non-maintenance anchor (b).</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="n"/>
+      <c r="E33" s="9" t="n"/>
+      <c r="F33" s="9" t="n"/>
+      <c r="G33" s="9" t="n"/>
+      <c r="H33" s="9" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_ALLO_LOT_FLG / LOTN_CART_LOT_FLG</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>No ALLO or CAR-T trigger.</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="n"/>
+      <c r="E34" s="9" t="n"/>
+      <c r="F34" s="9" t="n"/>
+      <c r="G34" s="9" t="n"/>
+      <c r="H34" s="9" t="n"/>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>WORKED EXAMPLE B - LOT2 starts on an allogeneic SCT</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="60" customHeight="1">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>Example B - LOT2 starts on an ALLOGENEIC SCT.
+Patient on VRd in LOT1 receives an allogeneic SCT on 2025-09-15. Per protocol, ALLO is its own LOT with no other MM therapies. LOT1 ends 2025-09-14 (day before ALLO). Next MM therapy after the ALLO date is daratumumab on 2025-12-10, which starts LOT3.</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="n"/>
+      <c r="C38" s="10" t="n"/>
+      <c r="D38" s="10" t="n"/>
+      <c r="E38" s="10" t="n"/>
+      <c r="F38" s="10" t="n"/>
+      <c r="G38" s="10" t="n"/>
+      <c r="H38" s="11" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>Value for this patient</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>How it was derived</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="n"/>
+      <c r="E39" s="12" t="n"/>
+      <c r="F39" s="12" t="n"/>
+      <c r="G39" s="12" t="n"/>
+      <c r="H39" s="12" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>LOT_NUM</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr"/>
+      <c r="D40" s="9" t="n"/>
+      <c r="E40" s="9" t="n"/>
+      <c r="F40" s="9" t="n"/>
+      <c r="G40" s="9" t="n"/>
+      <c r="H40" s="9" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_START_DT</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>2025-09-15</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>ALLO_DT (always starts a new LOT).</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="n"/>
+      <c r="E41" s="9" t="n"/>
+      <c r="F41" s="9" t="n"/>
+      <c r="G41" s="9" t="n"/>
+      <c r="H41" s="9" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_START_TYPE</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>SCT_ALLO</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr"/>
+      <c r="D42" s="9" t="n"/>
+      <c r="E42" s="9" t="n"/>
+      <c r="F42" s="9" t="n"/>
+      <c r="G42" s="9" t="n"/>
+      <c r="H42" s="9" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_MEDS</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>(empty)</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>ALLO LOT contains NO MM therapies.</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="n"/>
+      <c r="E43" s="9" t="n"/>
+      <c r="F43" s="9" t="n"/>
+      <c r="G43" s="9" t="n"/>
+      <c r="H43" s="9" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_MED_CNT</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr"/>
+      <c r="D44" s="9" t="n"/>
+      <c r="E44" s="9" t="n"/>
+      <c r="F44" s="9" t="n"/>
+      <c r="G44" s="9" t="n"/>
+      <c r="H44" s="9" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_ALLO_LOT_FLG</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Trigger type is SCT_ALLO.</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="n"/>
+      <c r="E45" s="9" t="n"/>
+      <c r="F45" s="9" t="n"/>
+      <c r="G45" s="9" t="n"/>
+      <c r="H45" s="9" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_END_DT (draft)</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>2025-09-15</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>Draft Q2 assumption: single-day LOT (start = end = ALLO_DT). Next agent (DARA on 2025-12-10) opens LOT3.</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="n"/>
+      <c r="E46" s="9" t="n"/>
+      <c r="F46" s="9" t="n"/>
+      <c r="G46" s="9" t="n"/>
+      <c r="H46" s="9" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_END_REASON</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>MED_ADD</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>DARA on 2025-12-10 is the next event; LOT2 ends the day before LOT3 starts. (Pending Q2.)</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="n"/>
+      <c r="E47" s="9" t="n"/>
+      <c r="F47" s="9" t="n"/>
+      <c r="G47" s="9" t="n"/>
+      <c r="H47" s="9" t="n"/>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>WORKED EXAMPLE C - LOT2 starts on an unplanned autologous SCT</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="60" customHeight="1">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>Example C - LOT2 starts on an UNPLANNED autologous SCT.
+Patient had a single AUTO during LOT1 on 2025-03-01. A second AUTO occurs on 2025-10-15 - 228 days later, which is &gt;180 days, so it is unplanned. The unplanned AUTO ends LOT1 (2025-10-14) and starts LOT2 on the AUTO date itself.</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="n"/>
+      <c r="C51" s="10" t="n"/>
+      <c r="D51" s="10" t="n"/>
+      <c r="E51" s="10" t="n"/>
+      <c r="F51" s="10" t="n"/>
+      <c r="G51" s="10" t="n"/>
+      <c r="H51" s="11" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="12" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>Value for this patient</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="inlineStr">
+        <is>
+          <t>How it was derived</t>
+        </is>
+      </c>
+      <c r="D52" s="12" t="n"/>
+      <c r="E52" s="12" t="n"/>
+      <c r="F52" s="12" t="n"/>
+      <c r="G52" s="12" t="n"/>
+      <c r="H52" s="12" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>LOT_NUM</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr"/>
+      <c r="D53" s="9" t="n"/>
+      <c r="E53" s="9" t="n"/>
+      <c r="F53" s="9" t="n"/>
+      <c r="G53" s="9" t="n"/>
+      <c r="H53" s="9" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_START_DT</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>Unplanned AUTO date (&gt;180d after prior AUTO).</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="n"/>
+      <c r="E54" s="9" t="n"/>
+      <c r="F54" s="9" t="n"/>
+      <c r="G54" s="9" t="n"/>
+      <c r="H54" s="9" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_START_TYPE</t>
+        </is>
+      </c>
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>SCT_AUTO</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>Unplanned AUTO is a first-class LOT-start trigger. (Planned tandem 60-180d would NOT start a new LOT.)</t>
+        </is>
+      </c>
+      <c r="D55" s="9" t="n"/>
+      <c r="E55" s="9" t="n"/>
+      <c r="F55" s="9" t="n"/>
+      <c r="G55" s="9" t="n"/>
+      <c r="H55" s="9" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="13" t="inlineStr">
+        <is>
+          <t>INDUCTION_WINDOW_DAYS</t>
+        </is>
+      </c>
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>LOT2 captures any post-AUTO agents within [2025-10-15, 2025-11-13].</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="n"/>
+      <c r="E56" s="9" t="n"/>
+      <c r="F56" s="9" t="n"/>
+      <c r="G56" s="9" t="n"/>
+      <c r="H56" s="9" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_TX_AUTO_FLG</t>
+        </is>
+      </c>
+      <c r="B57" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>AUTO occurred during LOT2.</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="n"/>
+      <c r="E57" s="9" t="n"/>
+      <c r="F57" s="9" t="n"/>
+      <c r="G57" s="9" t="n"/>
+      <c r="H57" s="9" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_TX_AUTO_SING_FLG</t>
+        </is>
+      </c>
+      <c r="B58" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
+        <is>
+          <t>Single AUTO during LOT2 (no second AUTO within tandem window).</t>
+        </is>
+      </c>
+      <c r="D58" s="9" t="n"/>
+      <c r="E58" s="9" t="n"/>
+      <c r="F58" s="9" t="n"/>
+      <c r="G58" s="9" t="n"/>
+      <c r="H58" s="9" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_TX_AUTO_TAND_FLG</t>
+        </is>
+      </c>
+      <c r="B59" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr"/>
+      <c r="D59" s="9" t="n"/>
+      <c r="E59" s="9" t="n"/>
+      <c r="F59" s="9" t="n"/>
+      <c r="G59" s="9" t="n"/>
+      <c r="H59" s="9" t="n"/>
+    </row>
   </sheetData>
+  <mergeCells count="36">
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C41:H41"/>
+    <mergeCell ref="C47:H47"/>
+    <mergeCell ref="C54:H54"/>
+    <mergeCell ref="C55:H55"/>
+    <mergeCell ref="C44:H44"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C40:H40"/>
+    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="C31:H31"/>
+    <mergeCell ref="C43:H43"/>
+    <mergeCell ref="C56:H56"/>
+    <mergeCell ref="C59:H59"/>
+    <mergeCell ref="C46:H46"/>
+    <mergeCell ref="C27:H27"/>
+    <mergeCell ref="C52:H52"/>
+    <mergeCell ref="C23:H23"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A50:H50"/>
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="C57:H57"/>
+    <mergeCell ref="C28:H28"/>
+    <mergeCell ref="C53:H53"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="C30:H30"/>
+    <mergeCell ref="C33:H33"/>
+    <mergeCell ref="C24:H24"/>
+    <mergeCell ref="C42:H42"/>
+    <mergeCell ref="C58:H58"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="C45:H45"/>
+    <mergeCell ref="C26:H26"/>
+    <mergeCell ref="C29:H29"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1591,7 +2614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2178,7 +3201,542 @@
       </c>
       <c r="H15" s="7" t="inlineStr"/>
     </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>WORKED EXAMPLE D - End-reason priority with CART_INIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Example D - END-REASON RESOLUTION (priority logic).
+LOT3 started 2025-11-01 with KRd. The patient has multiple competing end events:
+  - Run-out date of induction agents (DISCONTINUATION candidate): 2026-04-15
+  - First add med (POMA) on 2026-03-20 -&gt; LOT3 would end 2026-03-19 (MED_ADD)
+  - CAR-T infusion on 2026-04-02 (within 45 days of POMA)  -&gt; CART_INIT applies
+  - Death (YMDOD) on 2026-05-20
+Apply priority: SCT_ALLO &gt; SCT_CART &gt; SCT_AUTO &gt; CART_INIT &gt; MED_ADD &gt; DISCONTINUATION &gt; DEATH &gt; STUDY_END.</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
+      <c r="H19" s="11" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Value for this patient</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>How it was derived</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="n"/>
+      <c r="E20" s="12" t="n"/>
+      <c r="F20" s="12" t="n"/>
+      <c r="G20" s="12" t="n"/>
+      <c r="H20" s="12" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_END_DT</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>FIRST_CART_DT (2026-04-02) - 1. CART_INIT outranks MED_ADD because CAR-T occurred within 45d of the first add.</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="n"/>
+      <c r="E21" s="9" t="n"/>
+      <c r="F21" s="9" t="n"/>
+      <c r="G21" s="9" t="n"/>
+      <c r="H21" s="9" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_END_REASON</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>CART_INIT</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Highest-priority qualifying reason among competing events.</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="9" t="n"/>
+      <c r="F22" s="9" t="n"/>
+      <c r="G22" s="9" t="n"/>
+      <c r="H22" s="9" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_LENGTH</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>152</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-01 minus 2025-11-01 + 1 = 152 days.</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="n"/>
+      <c r="E23" s="9" t="n"/>
+      <c r="F23" s="9" t="n"/>
+      <c r="G23" s="9" t="n"/>
+      <c r="H23" s="9" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>LOT_(N+1)_START_DT</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>FIRST_CART_DT becomes LOT4 start; LOT4_START_TYPE = CART.</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="n"/>
+      <c r="E24" s="9" t="n"/>
+      <c r="F24" s="9" t="n"/>
+      <c r="G24" s="9" t="n"/>
+      <c r="H24" s="9" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_END_DT_CE_SENS</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Same as primary - no disenrollment cap binds earlier.</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="9" t="n"/>
+      <c r="F25" s="9" t="n"/>
+      <c r="G25" s="9" t="n"/>
+      <c r="H25" s="9" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_END_REASON_CE_SENS</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>CART_INIT</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr"/>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="9" t="n"/>
+      <c r="F26" s="9" t="n"/>
+      <c r="G26" s="9" t="n"/>
+      <c r="H26" s="9" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>WORKED EXAMPLE E - Discontinuation (run-out)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="60" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Example E - DISCONTINUATION (regimen runs out, no new agent within gap).
+LOT2 started 2025-08-20 with DARA + LENA. Last LENA fill (28-day supply) is 2026-01-10, MAP_END_DT = 2026-02-06. Last DARA infusion MAP_END_DT = 2026-01-15. No new MM agent appears in the next 90 days. Patient is alive and enrolled.</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="10" t="n"/>
+      <c r="E30" s="10" t="n"/>
+      <c r="F30" s="10" t="n"/>
+      <c r="G30" s="10" t="n"/>
+      <c r="H30" s="11" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>Value for this patient</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>How it was derived</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="12" t="n"/>
+      <c r="G31" s="12" t="n"/>
+      <c r="H31" s="12" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_DISCON_DT</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>max(MAP_END_DT) across LOT2 induction agents (the later LENA run-out).</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="n"/>
+      <c r="E32" s="9" t="n"/>
+      <c r="F32" s="9" t="n"/>
+      <c r="G32" s="9" t="n"/>
+      <c r="H32" s="9" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_END_DT</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>DISCONTINUATION uses the run-out date itself.</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="n"/>
+      <c r="E33" s="9" t="n"/>
+      <c r="F33" s="9" t="n"/>
+      <c r="G33" s="9" t="n"/>
+      <c r="H33" s="9" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_END_REASON</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>DISCONTINUATION</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>All agents reached run-out and no new agent within 90-day gap.</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="n"/>
+      <c r="E34" s="9" t="n"/>
+      <c r="F34" s="9" t="n"/>
+      <c r="G34" s="9" t="n"/>
+      <c r="H34" s="9" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_LENGTH</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>171</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>2026-02-06 minus 2025-08-20 + 1.</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="n"/>
+      <c r="E35" s="9" t="n"/>
+      <c r="F35" s="9" t="n"/>
+      <c r="G35" s="9" t="n"/>
+      <c r="H35" s="9" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>Next LOT?</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Only if a new MM agent eventually appears</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>If no further therapy, study/death/sensitivity will eventually close follow-up.</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="n"/>
+      <c r="E36" s="9" t="n"/>
+      <c r="F36" s="9" t="n"/>
+      <c r="G36" s="9" t="n"/>
+      <c r="H36" s="9" t="n"/>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>WORKED EXAMPLE F - Disenrollment primary vs sensitivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="60" customHeight="1">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>Example F - DISENROLLMENT: primary analysis vs sensitivity analysis.
+LOT4 started 2026-01-05. Patient disenrolls (ELIGEND) on 2026-04-30 with no death and no further therapy. study_end is 2026-12-31. This shows how the same patient produces different LOT4 closures under primary vs sensitivity.</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="n"/>
+      <c r="C40" s="10" t="n"/>
+      <c r="D40" s="10" t="n"/>
+      <c r="E40" s="10" t="n"/>
+      <c r="F40" s="10" t="n"/>
+      <c r="G40" s="10" t="n"/>
+      <c r="H40" s="11" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>Value for this patient</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>How it was derived</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="n"/>
+      <c r="E41" s="12" t="n"/>
+      <c r="F41" s="12" t="n"/>
+      <c r="G41" s="12" t="n"/>
+      <c r="H41" s="12" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_END_DT (PRIMARY)</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Disenrollment is IGNORED in primary; earliest of {death, study_end} = study_end.</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="n"/>
+      <c r="E42" s="9" t="n"/>
+      <c r="F42" s="9" t="n"/>
+      <c r="G42" s="9" t="n"/>
+      <c r="H42" s="9" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_END_REASON (PRIMARY)</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>STUDY_END</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>Primary analysis cannot use DISENROLLMENT.</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="n"/>
+      <c r="E43" s="9" t="n"/>
+      <c r="F43" s="9" t="n"/>
+      <c r="G43" s="9" t="n"/>
+      <c r="H43" s="9" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_END_DT_CE_SENS (SENSITIVITY)</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>ENDDATE_CE = min(YMDOD, ELIGEND, study_end) = ELIGEND.</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="n"/>
+      <c r="E44" s="9" t="n"/>
+      <c r="F44" s="9" t="n"/>
+      <c r="G44" s="9" t="n"/>
+      <c r="H44" s="9" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_END_REASON_CE_SENS (SENSITIVITY)</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>DISENROLLMENT</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Spec requires labelling DISENROLLMENT (do NOT collapse to STUDY_END).</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="n"/>
+      <c r="E45" s="9" t="n"/>
+      <c r="F45" s="9" t="n"/>
+      <c r="G45" s="9" t="n"/>
+      <c r="H45" s="9" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_LENGTH (PRIMARY)</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>361</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>2026-12-31 minus 2026-01-05 + 1.</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="n"/>
+      <c r="E46" s="9" t="n"/>
+      <c r="F46" s="9" t="n"/>
+      <c r="G46" s="9" t="n"/>
+      <c r="H46" s="9" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_LENGTH_CE_SENS</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>116</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-30 minus 2026-01-05 + 1.</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="n"/>
+      <c r="E47" s="9" t="n"/>
+      <c r="F47" s="9" t="n"/>
+      <c r="G47" s="9" t="n"/>
+      <c r="H47" s="9" t="n"/>
+    </row>
   </sheetData>
+  <mergeCells count="26">
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C41:H41"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="C47:H47"/>
+    <mergeCell ref="C44:H44"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C31:H31"/>
+    <mergeCell ref="C43:H43"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C46:H46"/>
+    <mergeCell ref="C36:H36"/>
+    <mergeCell ref="C23:H23"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="C33:H33"/>
+    <mergeCell ref="C24:H24"/>
+    <mergeCell ref="C42:H42"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="C45:H45"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="C35:H35"/>
+    <mergeCell ref="C26:H26"/>
+    <mergeCell ref="C20:H20"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3022,4 +4580,860 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AQ13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="3.2" customWidth="1" min="4" max="4"/>
+    <col width="3.2" customWidth="1" min="5" max="5"/>
+    <col width="3.2" customWidth="1" min="6" max="6"/>
+    <col width="3.2" customWidth="1" min="7" max="7"/>
+    <col width="3.2" customWidth="1" min="8" max="8"/>
+    <col width="3.2" customWidth="1" min="9" max="9"/>
+    <col width="3.2" customWidth="1" min="10" max="10"/>
+    <col width="3.2" customWidth="1" min="11" max="11"/>
+    <col width="3.2" customWidth="1" min="12" max="12"/>
+    <col width="3.2" customWidth="1" min="13" max="13"/>
+    <col width="3.2" customWidth="1" min="14" max="14"/>
+    <col width="3.2" customWidth="1" min="15" max="15"/>
+    <col width="3.2" customWidth="1" min="16" max="16"/>
+    <col width="3.2" customWidth="1" min="17" max="17"/>
+    <col width="3.2" customWidth="1" min="18" max="18"/>
+    <col width="3.2" customWidth="1" min="19" max="19"/>
+    <col width="3.2" customWidth="1" min="20" max="20"/>
+    <col width="3.2" customWidth="1" min="21" max="21"/>
+    <col width="3.2" customWidth="1" min="22" max="22"/>
+    <col width="3.2" customWidth="1" min="23" max="23"/>
+    <col width="3.2" customWidth="1" min="24" max="24"/>
+    <col width="3.2" customWidth="1" min="25" max="25"/>
+    <col width="3.2" customWidth="1" min="26" max="26"/>
+    <col width="3.2" customWidth="1" min="27" max="27"/>
+    <col width="3.2" customWidth="1" min="28" max="28"/>
+    <col width="3.2" customWidth="1" min="29" max="29"/>
+    <col width="3.2" customWidth="1" min="30" max="30"/>
+    <col width="3.2" customWidth="1" min="31" max="31"/>
+    <col width="3.2" customWidth="1" min="32" max="32"/>
+    <col width="3.2" customWidth="1" min="33" max="33"/>
+    <col width="3.2" customWidth="1" min="34" max="34"/>
+    <col width="3.2" customWidth="1" min="35" max="35"/>
+    <col width="3.2" customWidth="1" min="36" max="36"/>
+    <col width="3.2" customWidth="1" min="37" max="37"/>
+    <col width="3.2" customWidth="1" min="38" max="38"/>
+    <col width="3.2" customWidth="1" min="39" max="39"/>
+    <col width="3.2" customWidth="1" min="40" max="40"/>
+    <col width="3.2" customWidth="1" min="41" max="41"/>
+    <col width="3.2" customWidth="1" min="42" max="42"/>
+    <col width="3.2" customWidth="1" min="43" max="43"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Patient timelines (Gantt-style) - illustrating LOT2-5 transitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Legend:</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>LOT1</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>LOT2</t>
+        </is>
+      </c>
+      <c r="D2" s="18" t="inlineStr">
+        <is>
+          <t>LOT3</t>
+        </is>
+      </c>
+      <c r="E2" s="19" t="inlineStr">
+        <is>
+          <t>LOT4</t>
+        </is>
+      </c>
+      <c r="F2" s="20" t="inlineStr">
+        <is>
+          <t>LOT5</t>
+        </is>
+      </c>
+      <c r="G2" s="21" t="inlineStr">
+        <is>
+          <t>30d induction</t>
+        </is>
+      </c>
+      <c r="H2" s="22" t="inlineStr">
+        <is>
+          <t>AUTO SCT</t>
+        </is>
+      </c>
+      <c r="I2" s="23" t="inlineStr">
+        <is>
+          <t>ALLO SCT</t>
+        </is>
+      </c>
+      <c r="J2" s="24" t="inlineStr">
+        <is>
+          <t>CAR-T</t>
+        </is>
+      </c>
+      <c r="K2" s="25" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="L2" s="26" t="inlineStr">
+        <is>
+          <t>Med add</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>Day -&gt;</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="28" t="inlineStr"/>
+      <c r="F4" s="28" t="inlineStr"/>
+      <c r="G4" s="28" t="inlineStr"/>
+      <c r="H4" s="28" t="n">
+        <v>56</v>
+      </c>
+      <c r="I4" s="28" t="inlineStr"/>
+      <c r="J4" s="28" t="inlineStr"/>
+      <c r="K4" s="28" t="inlineStr"/>
+      <c r="L4" s="28" t="n">
+        <v>112</v>
+      </c>
+      <c r="M4" s="28" t="inlineStr"/>
+      <c r="N4" s="28" t="inlineStr"/>
+      <c r="O4" s="28" t="inlineStr"/>
+      <c r="P4" s="28" t="n">
+        <v>168</v>
+      </c>
+      <c r="Q4" s="28" t="inlineStr"/>
+      <c r="R4" s="28" t="inlineStr"/>
+      <c r="S4" s="28" t="inlineStr"/>
+      <c r="T4" s="28" t="n">
+        <v>224</v>
+      </c>
+      <c r="U4" s="28" t="inlineStr"/>
+      <c r="V4" s="28" t="inlineStr"/>
+      <c r="W4" s="28" t="inlineStr"/>
+      <c r="X4" s="28" t="n">
+        <v>280</v>
+      </c>
+      <c r="Y4" s="28" t="inlineStr"/>
+      <c r="Z4" s="28" t="inlineStr"/>
+      <c r="AA4" s="28" t="inlineStr"/>
+      <c r="AB4" s="28" t="n">
+        <v>336</v>
+      </c>
+      <c r="AC4" s="28" t="inlineStr"/>
+      <c r="AD4" s="28" t="inlineStr"/>
+      <c r="AE4" s="28" t="inlineStr"/>
+      <c r="AF4" s="28" t="n">
+        <v>392</v>
+      </c>
+      <c r="AG4" s="28" t="inlineStr"/>
+      <c r="AH4" s="28" t="inlineStr"/>
+      <c r="AI4" s="28" t="inlineStr"/>
+      <c r="AJ4" s="28" t="n">
+        <v>448</v>
+      </c>
+      <c r="AK4" s="28" t="inlineStr"/>
+      <c r="AL4" s="28" t="inlineStr"/>
+      <c r="AM4" s="28" t="inlineStr"/>
+      <c r="AN4" s="28" t="n">
+        <v>504</v>
+      </c>
+      <c r="AO4" s="28" t="inlineStr"/>
+      <c r="AP4" s="28" t="inlineStr"/>
+      <c r="AQ4" s="28" t="inlineStr"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>S1: LOT1 -&gt; LOT2 by MED_ADD</t>
+        </is>
+      </c>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>VRd LOT1; DARA added day 200 -&gt; LOT2 starts on DARA</t>
+        </is>
+      </c>
+      <c r="C5" s="30" t="inlineStr"/>
+      <c r="D5" s="31" t="inlineStr"/>
+      <c r="E5" s="31" t="inlineStr"/>
+      <c r="F5" s="31" t="inlineStr"/>
+      <c r="G5" s="31" t="inlineStr"/>
+      <c r="H5" s="31" t="inlineStr"/>
+      <c r="I5" s="32" t="inlineStr"/>
+      <c r="J5" s="32" t="inlineStr"/>
+      <c r="K5" s="32" t="inlineStr"/>
+      <c r="L5" s="32" t="inlineStr"/>
+      <c r="M5" s="32" t="inlineStr"/>
+      <c r="N5" s="32" t="inlineStr"/>
+      <c r="O5" s="32" t="inlineStr"/>
+      <c r="P5" s="32" t="inlineStr"/>
+      <c r="Q5" s="32" t="inlineStr"/>
+      <c r="R5" s="33" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="S5" s="34" t="inlineStr"/>
+      <c r="T5" s="34" t="inlineStr"/>
+      <c r="U5" s="35" t="inlineStr"/>
+      <c r="V5" s="35" t="inlineStr"/>
+      <c r="W5" s="35" t="inlineStr"/>
+      <c r="X5" s="35" t="inlineStr"/>
+      <c r="Y5" s="35" t="inlineStr"/>
+      <c r="Z5" s="35" t="inlineStr"/>
+      <c r="AA5" s="35" t="inlineStr"/>
+      <c r="AB5" s="35" t="inlineStr"/>
+      <c r="AC5" s="35" t="inlineStr"/>
+      <c r="AD5" s="35" t="inlineStr"/>
+      <c r="AE5" s="35" t="inlineStr"/>
+      <c r="AF5" s="35" t="inlineStr"/>
+      <c r="AG5" s="35" t="inlineStr"/>
+      <c r="AH5" s="35" t="inlineStr"/>
+      <c r="AI5" s="35" t="inlineStr"/>
+      <c r="AJ5" s="35" t="inlineStr"/>
+      <c r="AK5" s="35" t="inlineStr"/>
+      <c r="AL5" s="35" t="inlineStr"/>
+      <c r="AM5" s="35" t="inlineStr"/>
+      <c r="AN5" s="35" t="inlineStr"/>
+      <c r="AO5" s="35" t="inlineStr"/>
+      <c r="AP5" s="35" t="inlineStr"/>
+      <c r="AQ5" s="30" t="inlineStr"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>S2: LOT1 -&gt; LOT2 by unplanned AUTO</t>
+        </is>
+      </c>
+      <c r="B6" s="29" t="inlineStr">
+        <is>
+          <t>Single AUTO d100; second AUTO d320 (&gt;180d) is unplanned -&gt; LOT2 starts d320</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr"/>
+      <c r="D6" s="32" t="inlineStr"/>
+      <c r="E6" s="32" t="inlineStr"/>
+      <c r="F6" s="32" t="inlineStr"/>
+      <c r="G6" s="32" t="inlineStr"/>
+      <c r="H6" s="32" t="inlineStr"/>
+      <c r="I6" s="32" t="inlineStr"/>
+      <c r="J6" s="32" t="inlineStr"/>
+      <c r="K6" s="36" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L6" s="32" t="inlineStr"/>
+      <c r="M6" s="32" t="inlineStr"/>
+      <c r="N6" s="32" t="inlineStr"/>
+      <c r="O6" s="32" t="inlineStr"/>
+      <c r="P6" s="32" t="inlineStr"/>
+      <c r="Q6" s="32" t="inlineStr"/>
+      <c r="R6" s="32" t="inlineStr"/>
+      <c r="S6" s="32" t="inlineStr"/>
+      <c r="T6" s="32" t="inlineStr"/>
+      <c r="U6" s="32" t="inlineStr"/>
+      <c r="V6" s="32" t="inlineStr"/>
+      <c r="W6" s="32" t="inlineStr"/>
+      <c r="X6" s="32" t="inlineStr"/>
+      <c r="Y6" s="32" t="inlineStr"/>
+      <c r="Z6" s="37" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AA6" s="34" t="inlineStr"/>
+      <c r="AB6" s="34" t="inlineStr"/>
+      <c r="AC6" s="35" t="inlineStr"/>
+      <c r="AD6" s="35" t="inlineStr"/>
+      <c r="AE6" s="35" t="inlineStr"/>
+      <c r="AF6" s="35" t="inlineStr"/>
+      <c r="AG6" s="35" t="inlineStr"/>
+      <c r="AH6" s="35" t="inlineStr"/>
+      <c r="AI6" s="35" t="inlineStr"/>
+      <c r="AJ6" s="35" t="inlineStr"/>
+      <c r="AK6" s="35" t="inlineStr"/>
+      <c r="AL6" s="35" t="inlineStr"/>
+      <c r="AM6" s="35" t="inlineStr"/>
+      <c r="AN6" s="35" t="inlineStr"/>
+      <c r="AO6" s="35" t="inlineStr"/>
+      <c r="AP6" s="35" t="inlineStr"/>
+      <c r="AQ6" s="30" t="inlineStr"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>S3: LOT1 -&gt; LOT2 (ALLO LOT) -&gt; LOT3</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>ALLO d250 = LOT2 (1-day LOT, no MM); next agent d340 starts LOT3</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr"/>
+      <c r="D7" s="32" t="inlineStr"/>
+      <c r="E7" s="32" t="inlineStr"/>
+      <c r="F7" s="32" t="inlineStr"/>
+      <c r="G7" s="32" t="inlineStr"/>
+      <c r="H7" s="32" t="inlineStr"/>
+      <c r="I7" s="32" t="inlineStr"/>
+      <c r="J7" s="32" t="inlineStr"/>
+      <c r="K7" s="32" t="inlineStr"/>
+      <c r="L7" s="32" t="inlineStr"/>
+      <c r="M7" s="32" t="inlineStr"/>
+      <c r="N7" s="32" t="inlineStr"/>
+      <c r="O7" s="32" t="inlineStr"/>
+      <c r="P7" s="32" t="inlineStr"/>
+      <c r="Q7" s="32" t="inlineStr"/>
+      <c r="R7" s="32" t="inlineStr"/>
+      <c r="S7" s="32" t="inlineStr"/>
+      <c r="T7" s="32" t="inlineStr"/>
+      <c r="U7" s="38" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="V7" s="30" t="inlineStr"/>
+      <c r="W7" s="30" t="inlineStr"/>
+      <c r="X7" s="30" t="inlineStr"/>
+      <c r="Y7" s="30" t="inlineStr"/>
+      <c r="Z7" s="30" t="inlineStr"/>
+      <c r="AA7" s="30" t="inlineStr"/>
+      <c r="AB7" s="39" t="inlineStr"/>
+      <c r="AC7" s="39" t="inlineStr"/>
+      <c r="AD7" s="39" t="inlineStr"/>
+      <c r="AE7" s="40" t="inlineStr"/>
+      <c r="AF7" s="40" t="inlineStr"/>
+      <c r="AG7" s="40" t="inlineStr"/>
+      <c r="AH7" s="40" t="inlineStr"/>
+      <c r="AI7" s="40" t="inlineStr"/>
+      <c r="AJ7" s="40" t="inlineStr"/>
+      <c r="AK7" s="40" t="inlineStr"/>
+      <c r="AL7" s="40" t="inlineStr"/>
+      <c r="AM7" s="40" t="inlineStr"/>
+      <c r="AN7" s="40" t="inlineStr"/>
+      <c r="AO7" s="40" t="inlineStr"/>
+      <c r="AP7" s="40" t="inlineStr"/>
+      <c r="AQ7" s="30" t="inlineStr"/>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>S4: LOT1 -&gt; LOT2 (CAR-T LOT)</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="inlineStr">
+        <is>
+          <t>CAR-T d220; agents within 45d are consolidated into LOT2</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr"/>
+      <c r="D8" s="32" t="inlineStr"/>
+      <c r="E8" s="32" t="inlineStr"/>
+      <c r="F8" s="32" t="inlineStr"/>
+      <c r="G8" s="32" t="inlineStr"/>
+      <c r="H8" s="32" t="inlineStr"/>
+      <c r="I8" s="32" t="inlineStr"/>
+      <c r="J8" s="32" t="inlineStr"/>
+      <c r="K8" s="32" t="inlineStr"/>
+      <c r="L8" s="32" t="inlineStr"/>
+      <c r="M8" s="32" t="inlineStr"/>
+      <c r="N8" s="32" t="inlineStr"/>
+      <c r="O8" s="32" t="inlineStr"/>
+      <c r="P8" s="32" t="inlineStr"/>
+      <c r="Q8" s="32" t="inlineStr"/>
+      <c r="R8" s="32" t="inlineStr"/>
+      <c r="S8" s="41" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="T8" s="34" t="inlineStr"/>
+      <c r="U8" s="34" t="inlineStr"/>
+      <c r="V8" s="34" t="inlineStr"/>
+      <c r="W8" s="35" t="inlineStr"/>
+      <c r="X8" s="35" t="inlineStr"/>
+      <c r="Y8" s="35" t="inlineStr"/>
+      <c r="Z8" s="35" t="inlineStr"/>
+      <c r="AA8" s="35" t="inlineStr"/>
+      <c r="AB8" s="35" t="inlineStr"/>
+      <c r="AC8" s="35" t="inlineStr"/>
+      <c r="AD8" s="35" t="inlineStr"/>
+      <c r="AE8" s="35" t="inlineStr"/>
+      <c r="AF8" s="35" t="inlineStr"/>
+      <c r="AG8" s="35" t="inlineStr"/>
+      <c r="AH8" s="35" t="inlineStr"/>
+      <c r="AI8" s="35" t="inlineStr"/>
+      <c r="AJ8" s="35" t="inlineStr"/>
+      <c r="AK8" s="35" t="inlineStr"/>
+      <c r="AL8" s="35" t="inlineStr"/>
+      <c r="AM8" s="35" t="inlineStr"/>
+      <c r="AN8" s="35" t="inlineStr"/>
+      <c r="AO8" s="35" t="inlineStr"/>
+      <c r="AP8" s="35" t="inlineStr"/>
+      <c r="AQ8" s="30" t="inlineStr"/>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>S5: LOT2 -&gt; LOT3 by DISCONTINUATION + new agent</t>
+        </is>
+      </c>
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>LOT2 runs out d260; new agent d460 -&gt; LOT3</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr"/>
+      <c r="D9" s="32" t="inlineStr"/>
+      <c r="E9" s="32" t="inlineStr"/>
+      <c r="F9" s="32" t="inlineStr"/>
+      <c r="G9" s="32" t="inlineStr"/>
+      <c r="H9" s="32" t="inlineStr"/>
+      <c r="I9" s="32" t="inlineStr"/>
+      <c r="J9" s="32" t="inlineStr"/>
+      <c r="K9" s="32" t="inlineStr"/>
+      <c r="L9" s="32" t="inlineStr"/>
+      <c r="M9" s="32" t="inlineStr"/>
+      <c r="N9" s="32" t="inlineStr"/>
+      <c r="O9" s="32" t="inlineStr"/>
+      <c r="P9" s="32" t="inlineStr"/>
+      <c r="Q9" s="32" t="inlineStr"/>
+      <c r="R9" s="34" t="inlineStr"/>
+      <c r="S9" s="34" t="inlineStr"/>
+      <c r="T9" s="34" t="inlineStr"/>
+      <c r="U9" s="35" t="inlineStr"/>
+      <c r="V9" s="35" t="inlineStr"/>
+      <c r="W9" s="30" t="inlineStr"/>
+      <c r="X9" s="30" t="inlineStr"/>
+      <c r="Y9" s="30" t="inlineStr"/>
+      <c r="Z9" s="30" t="inlineStr"/>
+      <c r="AA9" s="30" t="inlineStr"/>
+      <c r="AB9" s="30" t="inlineStr"/>
+      <c r="AC9" s="30" t="inlineStr"/>
+      <c r="AD9" s="30" t="inlineStr"/>
+      <c r="AE9" s="30" t="inlineStr"/>
+      <c r="AF9" s="30" t="inlineStr"/>
+      <c r="AG9" s="30" t="inlineStr"/>
+      <c r="AH9" s="30" t="inlineStr"/>
+      <c r="AI9" s="30" t="inlineStr"/>
+      <c r="AJ9" s="39" t="inlineStr"/>
+      <c r="AK9" s="39" t="inlineStr"/>
+      <c r="AL9" s="39" t="inlineStr"/>
+      <c r="AM9" s="40" t="inlineStr"/>
+      <c r="AN9" s="40" t="inlineStr"/>
+      <c r="AO9" s="40" t="inlineStr"/>
+      <c r="AP9" s="40" t="inlineStr"/>
+      <c r="AQ9" s="30" t="inlineStr"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>S6: LOT3 ends by DEATH</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="inlineStr">
+        <is>
+          <t>Death d420 closes LOT3; no LOT4</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr"/>
+      <c r="D10" s="32" t="inlineStr"/>
+      <c r="E10" s="32" t="inlineStr"/>
+      <c r="F10" s="32" t="inlineStr"/>
+      <c r="G10" s="32" t="inlineStr"/>
+      <c r="H10" s="32" t="inlineStr"/>
+      <c r="I10" s="32" t="inlineStr"/>
+      <c r="J10" s="32" t="inlineStr"/>
+      <c r="K10" s="32" t="inlineStr"/>
+      <c r="L10" s="32" t="inlineStr"/>
+      <c r="M10" s="32" t="inlineStr"/>
+      <c r="N10" s="32" t="inlineStr"/>
+      <c r="O10" s="32" t="inlineStr"/>
+      <c r="P10" s="32" t="inlineStr"/>
+      <c r="Q10" s="32" t="inlineStr"/>
+      <c r="R10" s="35" t="inlineStr"/>
+      <c r="S10" s="35" t="inlineStr"/>
+      <c r="T10" s="35" t="inlineStr"/>
+      <c r="U10" s="35" t="inlineStr"/>
+      <c r="V10" s="35" t="inlineStr"/>
+      <c r="W10" s="35" t="inlineStr"/>
+      <c r="X10" s="35" t="inlineStr"/>
+      <c r="Y10" s="35" t="inlineStr"/>
+      <c r="Z10" s="35" t="inlineStr"/>
+      <c r="AA10" s="35" t="inlineStr"/>
+      <c r="AB10" s="40" t="inlineStr"/>
+      <c r="AC10" s="40" t="inlineStr"/>
+      <c r="AD10" s="40" t="inlineStr"/>
+      <c r="AE10" s="40" t="inlineStr"/>
+      <c r="AF10" s="40" t="inlineStr"/>
+      <c r="AG10" s="40" t="inlineStr"/>
+      <c r="AH10" s="42" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="AI10" s="30" t="inlineStr"/>
+      <c r="AJ10" s="30" t="inlineStr"/>
+      <c r="AK10" s="30" t="inlineStr"/>
+      <c r="AL10" s="30" t="inlineStr"/>
+      <c r="AM10" s="30" t="inlineStr"/>
+      <c r="AN10" s="30" t="inlineStr"/>
+      <c r="AO10" s="30" t="inlineStr"/>
+      <c r="AP10" s="30" t="inlineStr"/>
+      <c r="AQ10" s="30" t="inlineStr"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>S7: Tandem AUTO during LOT2 (NO new LOT)</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>AUTO d250 then AUTO d340 (90d apart, planned tandem) - LOT2 continues</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr"/>
+      <c r="D11" s="32" t="inlineStr"/>
+      <c r="E11" s="32" t="inlineStr"/>
+      <c r="F11" s="32" t="inlineStr"/>
+      <c r="G11" s="32" t="inlineStr"/>
+      <c r="H11" s="32" t="inlineStr"/>
+      <c r="I11" s="32" t="inlineStr"/>
+      <c r="J11" s="32" t="inlineStr"/>
+      <c r="K11" s="32" t="inlineStr"/>
+      <c r="L11" s="32" t="inlineStr"/>
+      <c r="M11" s="32" t="inlineStr"/>
+      <c r="N11" s="32" t="inlineStr"/>
+      <c r="O11" s="32" t="inlineStr"/>
+      <c r="P11" s="32" t="inlineStr"/>
+      <c r="Q11" s="32" t="inlineStr"/>
+      <c r="R11" s="34" t="inlineStr"/>
+      <c r="S11" s="34" t="inlineStr"/>
+      <c r="T11" s="34" t="inlineStr"/>
+      <c r="U11" s="36" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="V11" s="35" t="inlineStr"/>
+      <c r="W11" s="35" t="inlineStr"/>
+      <c r="X11" s="35" t="inlineStr"/>
+      <c r="Y11" s="35" t="inlineStr"/>
+      <c r="Z11" s="35" t="inlineStr"/>
+      <c r="AA11" s="35" t="inlineStr"/>
+      <c r="AB11" s="36" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="AC11" s="35" t="inlineStr"/>
+      <c r="AD11" s="35" t="inlineStr"/>
+      <c r="AE11" s="35" t="inlineStr"/>
+      <c r="AF11" s="35" t="inlineStr"/>
+      <c r="AG11" s="35" t="inlineStr"/>
+      <c r="AH11" s="35" t="inlineStr"/>
+      <c r="AI11" s="35" t="inlineStr"/>
+      <c r="AJ11" s="35" t="inlineStr"/>
+      <c r="AK11" s="35" t="inlineStr"/>
+      <c r="AL11" s="35" t="inlineStr"/>
+      <c r="AM11" s="35" t="inlineStr"/>
+      <c r="AN11" s="35" t="inlineStr"/>
+      <c r="AO11" s="35" t="inlineStr"/>
+      <c r="AP11" s="35" t="inlineStr"/>
+      <c r="AQ11" s="30" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Each cell = ~14 days. Markers: M=Med add, A=AUTO SCT, X=ALLO SCT, C=CAR-T, +=Death. Yellow top edge = induction window overlay. Single-cell-only LOT = singleton ALLO LOT (Q2 draft assumption).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A13:AQ13"/>
+    <mergeCell ref="A1:R1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Decision flow: when does LOT(N+1) start?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Read top-to-bottom. Each event evaluates AFTER LOT_N_BASE_END_DT. The earliest qualifying trigger determines LOT_(N+1)_START_DT and LOTN+1_START_TYPE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>If YES</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>If NO -&gt; next step</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Is there an ALLO SCT after LOT_N ended?</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>LOT_(N+1) starts at ALLO_DT. LOTN+1_START_TYPE = SCT_ALLO. ALLO LOT contains NO MM therapies.</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Step 2</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>ALLO always wins ties on the same day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Is there a CAR-T infusion after LOT_N ended?</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>LOT_(N+1) starts at FIRST_CART_DT. LOTN+1_START_TYPE = CART. Agents within 45d are consolidated (Apr 22 decision).</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Step 3</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>CAR-T outranks AUTO and MED on tie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Is there an UNPLANNED AUTO SCT after LOT_N ended?
+(&gt;180d after the prior AUTO in LOT_N, OR an isolated AUTO in a new line)</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>LOT_(N+1) starts at AUTO_DT. LOTN+1_START_TYPE = SCT_AUTO.</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Step 4</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Planned/single/tandem AUTO within 60-180d of a prior AUTO is a CONTINUATION - it does NOT start a new LOT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Is there a new MM oncology agent (non-steroid, non-permissible-substitute) after LOT_N ended?</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>LOT_(N+1) starts at MAP_START_DT of that agent. LOTN+1_START_TYPE = MED.</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Step 5</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Steroids alone do NOT start a LOT. Biosimilar substitutions do NOT start a LOT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Has DEATH (YMDOD) or STUDY_END been reached?</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Follow-up ends. No LOT_(N+1).</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Step 6 (sensitivity)</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>PRIMARY analysis closes here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>SENSITIVITY ONLY: is CENSOR_AT_DISENROLLMENT = TRUE and ELIGEND earliest?</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Sensitivity output caps at ENDDATE_CE; LOTN_BASE_END_REASON_CE_SENS = DISENROLLMENT.</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>End</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Primary analysis ignores ELIGEND. See Q12.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="50" customHeight="1">
+      <c r="A12" s="43" t="inlineStr">
+        <is>
+          <t>Same-day tie-break priority (highest wins): SCT_ALLO &gt; SCT_CART &gt; SCT_AUTO (unplanned) &gt; CART_INIT &gt; MED_ADD &gt; DISCONTINUATION &gt; DEATH &gt; STUDY_END (PRIMARY); DISENROLLMENT slots between DEATH and STUDY_END in SENSITIVITY only.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A12:E12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
LOT2-5 spec: tighten verbose definitions; flag inherited assumptions
- Cut definitions/notes throughout: LOTN_START_DT, LOTN_BASE_MEDS,
  dynamic flag rows, LOTN_END_DT_TEMP, end-reason/length rows, examples,
  scenarios, and trigger-sheet rows. Verbose-cell count dropped from 30
  to 4.
- Flag as DRAFT/inherits-LOT1 (not asserted as fact) the same-day
  tie-break priority, the CART_INIT 45d-of-first-add rule for LOT2-5,
  and the LOTN_TX_ vs LOTN_SCT_ flag prefix. New Q13 (prefix) and Q14
  (priority order) added to Open_Questions.
- Fix imprecise wording in LOTN_BASE_END_DT_CE_SENS variable definition
  ('cap at ELIGEND' rather than 'min(YMDOD, ELIGEND, study_end)' which
  conflated the cap with the full end-date logic).
</commit_message>
<xml_diff>
--- a/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
+++ b/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
@@ -738,7 +738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -784,295 +784,283 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>DRAFT - first stab; for QC by Julia</t>
+          <t>DRAFT - first stab; for QC</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Author</t>
+          <t>Draft Date</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Onkar (Claude-assisted draft)</t>
+          <t>30-Apr-2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Draft Date</t>
+          <t>Source Protocol</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>30-Apr-2026</t>
+          <t>Lot protocol Apr 13.pdf (v6)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Source Protocol</t>
+          <t>Parent Spec</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Lot protocol Apr 13.pdf (v6 of LOT rules)</t>
+          <t>lot1baseapr18.pdf / lot1baseendupdatedapr19.pdf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Parent Spec</t>
+          <t>Reference</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>lot1baseapr18.pdf / lot1baseendupdatedapr19.pdf</t>
+          <t>Apr 22 meeting minutes</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Key reference</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Meeting Minutes Apr 22 (induction=30d; SCT/CAR-T can start LOT2-5)</t>
-        </is>
-      </c>
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr"/>
-      <c r="B11" s="3" t="inlineStr"/>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Tabs</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Tabs</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>1.Cover</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>This page</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>1.Cover</t>
+          <t>2.QC Review</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>This page</t>
+          <t>QC sign-off log</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2.QC Review</t>
+          <t>3.LOT2_5_BASE</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>QC sign-off log</t>
+          <t>LOT 2-5 base period definition (start, induction, regimen)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>3.LOT2_5_BASE</t>
+          <t>4.LOT2_5_BASE_END</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>LOT 2-5 base period definition (start, induction, regimen)</t>
+          <t>LOT 2-5 base end date and end reason derivation</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>4.LOT2_5_BASE_END</t>
+          <t>5.SCT_CART_LOT_START</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>LOT 2-5 base end date and end reason derivation</t>
+          <t>Rules for SCT/ALLO/CAR-T as LOT 2-5 starting events</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>5.SCT_CART_LOT_START</t>
+          <t>6.Scenarios</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Rules for SCT/ALLO/CAR-T as LOT 2-5 starting events</t>
+          <t>Worked scenarios LOT2-LOT5</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>6.Scenarios</t>
+          <t>7.Open_Questions</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Worked scenarios LOT2-LOT5</t>
+          <t>Items needing Julia's review</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>7.Open_Questions</t>
+          <t>8.Timelines</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Items needing Julia's review</t>
+          <t>Gantt-style patient journey examples (visual)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>8.Timelines</t>
+          <t>9.Decision_Flow</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Gantt-style patient journey examples (visual)</t>
+          <t>Decision tree for when LOT(N+1) starts</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>9.Decision_Flow</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Decision tree for when LOT(N+1) starts</t>
-        </is>
-      </c>
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr"/>
-      <c r="B22" s="3" t="inlineStr"/>
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Key differences vs LOT1</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Key differences vs LOT1</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Induction window</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>30d (LOT1 = 60d)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Induction window</t>
+          <t>LOT start trigger</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>30 days (vs 60 days for LOT1)</t>
+          <t>Earliest of: new MM agent / ALLO SCT / CAR-T / unplanned AUTO</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>LOT start trigger</t>
+          <t>Numbering</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>First MM oncology agent OR ALLO SCT OR CAR-T event (vs LOT1 = first MM agent only)</t>
+          <t>LOT_NUM = 2..5</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Numbering</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>LOT_NUM increments 2..5; same algorithmic rules otherwise</t>
+          <t>contains_mtx_reg flag only; no standalone maintenance LOT (inherits LOT1 code). Q5.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Steroids</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Follows current LOT1 CODE behaviour (descriptive contains_mtx_reg flag; no standalone maintenance LOT). Diverges from the protocol Rule 8 wording. Open Q5.</t>
+          <t>Excluded from regimen.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Permissible subs</t>
+          <t>Biosimilar subs</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Same as LOT1 - do not advance LOT</t>
+          <t>Do not advance LOT.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Steroids</t>
+          <t>CAR-T consolidation</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Excluded from regimen identification (per LOT1 protocol Section 5.1.1)</t>
+          <t>45d (Apr 22 decision; Q11 resolved).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>CAR-T consolidation</t>
+          <t>Disenrollment</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>45 days (per Apr 22 study-team decision; supersedes 30-day older protocol text). Resolved Q11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Disenrollment</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>PRIMARY analysis: ignored. SENSITIVITY (CENSOR_AT_DISENROLLMENT=TRUE) caps via ENDDATE_CE and emits DISENROLLMENT reason. Resolved Q12.</t>
+          <t>PRIMARY: ignored. SENSITIVITY: ENDDATE_CE cap, reason = DISENROLLMENT (Q12 resolved).</t>
         </is>
       </c>
     </row>
@@ -1316,17 +1304,17 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>LOTN_START_DT is the EARLIEST of any of the following competing triggers occurring after LOT_(N-1)_BASE_END_DT: (a) first MM oncology agent (non-steroid) administered/dispensed; (b) first UNPLANNED autologous SCT (AUTO) - i.e., an AUTO occurring &gt;180 days after a prior AUTO in LOT_(N-1). Planned, single, or tandem AUTO SCTs (60-180 day intervals) are continuations of the same LOT and do NOT trigger a new LOT; (c) first allogeneic SCT (ALLO) - ALLO always starts a new LOT; (d) first CAR-T infusion - CAR-T is classified as its own LOT. When LOT_(N-1) ended due to SCT_ALLO / SCT_CART / SCT_AUTO unplanned / CART_INIT, LOTN_START_DT equals the SCT or CAR-T event date itself (LOT_(N-1) ended the day before that event).</t>
+          <t>Earliest of, after LOT_(N-1)_BASE_END_DT: (a) first non-steroid MM oncology agent; (b) first ALLO SCT; (c) first CAR-T infusion; (d) first UNPLANNED AUTO SCT (&gt;180d after a prior AUTO). Planned/single/tandem AUTO is a continuation, not a trigger. Permissible biosimilar substitutions do not trigger.</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>CL_MMA_CODELIST (Tab 41), CL_SCT_CODELIST (Tab 44), CL_MMA_ROLLUP (Tab 40)</t>
+          <t>CL_MMA_CODELIST, CL_SCT_CODELIST, CL_MMA_ROLLUP</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>Source: T_MEDICAL (PROC_CD, BILL_PROC_CD, NDC), T_RX (NDC), T_MEDICAL procedure codes for SCT/CAR-T. Steroids excluded from medication-trigger candidates (MAP_MED_CLASS != 'STEROID'). Permissible biosimilar substitutions do NOT trigger a new LOT.</t>
+          <t>Source: T_MEDICAL (PROC_CD, BILL_PROC_CD, NDC), T_RX (NDC). Steroids excluded (MAP_MED_CLASS != 'STEROID').</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr"/>
@@ -1344,7 +1332,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Type of LOT N start event</t>
+          <t>Trigger that started LOT N</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -1354,7 +1342,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Indicates which trigger started LOT N: a new MM medication, an unplanned autologous SCT, an allogeneic SCT, or a CAR-T infusion. All four are first-class competing triggers - whichever is earliest defines LOTN_START_DT and LOTN_START_TYPE.</t>
+          <t>Type of the earliest qualifying trigger.</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -1364,7 +1352,7 @@
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>Determined from the event class on LOTN_START_DT. If multiple events on same day, priority: SCT_ALLO &gt; CART &gt; SCT_AUTO &gt; MED.</t>
+          <t>Same-day tie-break (DRAFT, inherits LOT1 - confirm): SCT_ALLO &gt; CART &gt; SCT_AUTO &gt; MED.</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr"/>
@@ -1382,17 +1370,17 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Induction regimen identification window</t>
+          <t>Induction window</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>30 (LOT2-5)</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Per protocol: 'For LOT2-LOT5, the LOT regimen includes all MM therapies received within 30 days on and following the LOT start date.' (Contrast: LOT1 uses 60 days.)</t>
+          <t>Window for identifying LOT N regimen. (LOT1 uses 60.)</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -1402,7 +1390,7 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Applied to MAP_START_DT from T_MEDICAL/T_RX claims. Medications with MAP_START_DT within [LOTN_START_DT, LOTN_START_DT + 29] inclusive are induction.</t>
+          <t>MAP_START_DT in [LOTN_START_DT, LOTN_START_DT + 29] = induction.</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr"/>
@@ -1425,22 +1413,22 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Comma-separated MED_ABBR list</t>
+          <t>Comma list of MED_ABBR</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>All MM oncology therapies received on and within 30 days of LOTN_START_DT, with the first therapy considered induction. Excludes corticosteroids (non-oncology supportive agents). Switches between a biologic reference product and its biosimilar(s), or between biosimilars of the same reference product, are permitted and do not constitute a change in regimen.</t>
+          <t>Non-steroid MM oncology agents within the 30-day induction window. Permissible biosimilar substitutions do not advance the regimen.</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>CL_MMA_CODELIST (Tab 41), CL_MMA_ROLLUP (Tab 40)</t>
+          <t>CL_MMA_CODELIST, CL_MMA_ROLLUP</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Filter MAP_MED_CLASS != 'STEROID'. Source: T_MEDICAL/T_RX matched to CL_MMA_CODELIST; abbreviation from CL_MMA_ROLLUP. Window: MAP_START_DT in [LOTN_START_DT, LOTN_START_DT + 29].</t>
+          <t>Filter MAP_MED_CLASS != 'STEROID'.</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr"/>
@@ -1458,7 +1446,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Count of distinct induction agents</t>
+          <t>Distinct induction agents</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -1468,7 +1456,7 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Number of unique non-steroid MM medication abbreviations in LOTN_BASE_MEDS.</t>
+          <t>Count of distinct MED_ABBR in LOTN_BASE_MEDS.</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -1476,11 +1464,7 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>Count distinct MED_ABBR within induction window.</t>
-        </is>
-      </c>
+      <c r="G7" s="7" t="inlineStr"/>
       <c r="H7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -1496,7 +1480,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Per-medication induction flags (one column per MED_ABBR)</t>
+          <t>Per-medication induction flags</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -1506,17 +1490,17 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>For each distinct medication abbreviation in CL_MMA_ROLLUP (Tab 40), emit a flag column LOTN_MED_BORT, LOTN_MED_LENA, LOTN_MED_DARA, LOTN_MED_CARF, LOTN_MED_IXAZ, LOTN_MED_THAL, LOTN_MED_POMA, LOTN_MED_CYCL, LOTN_MED_MELP, LOTN_MED_BEND, LOTN_MED_IDEC, LOTN_MED_CILT, LOTN_MED_BELA, LOTN_MED_ISAT, LOTN_MED_ELOT, LOTN_MED_ETOP, LOTN_MED_PANO, LOTN_MED_SELI, LOTN_MED_TECL, LOTN_MED_DOPL, LOTN_MED_DOXO, LOTN_MED_CISP, LOTN_MED_ELRA, LOTN_MED_LINV, LOTN_MED_TALQ, LOTN_MED_VENE, etc. = 1 if that medication is part of LOTN_BASE_MEDS.</t>
+          <t>One flag column per non-steroid MED_ABBR in CL_MMA_ROLLUP (e.g. LOTN_MED_BORT, LOTN_MED_LENA, LOTN_MED_DARA, ...). = 1 if that medication is in LOTN_BASE_MEDS.</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>CL_MMA_ROLLUP (Tab 40), CL_MMA_CODELIST (Tab 41)</t>
+          <t>CL_MMA_ROLLUP</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Mirror LOT1 dynamic flag generation. Steroid abbreviations (DEXA, PRED) excluded since regimen excludes steroids.</t>
+          <t>Mirror LOT1 dynamic flag generation; steroid abbreviations excluded.</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr"/>
@@ -1534,7 +1518,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Per-class induction flags (one column per MED_CLASS)</t>
+          <t>Per-class induction flags</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -1544,17 +1528,17 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>For each MED_CLASS in CL_MMA_ROLLUP, emit a flag column: LOTN_CLASS_PROTINHIB, LOTN_CLASS_IMMUNOMOD, LOTN_CLASS_ANTICD38, LOTN_CLASS_BCMA, LOTN_CLASS_MUSTARD, LOTN_CLASS_SIGNALING, LOTN_CLASS_TOPOISOMERASE, LOTN_CLASS_HDACINHIBITOR, LOTN_CLASS_XPORTINHIBITOR, LOTN_CLASS_ANTHRACYCLINE, LOTN_CLASS_PLATINUM, LOTN_CLASS_CELMOD, LOTN_CLASS_BCL2INHIBITOR. = 1 if any agent of that class is in LOTN_BASE_MEDS.</t>
+          <t>One flag column per non-steroid MED_CLASS in CL_MMA_ROLLUP (e.g. LOTN_CLASS_PROTINHIB, LOTN_CLASS_IMMUNOMOD, ...). = 1 if any LOTN_BASE_MEDS agent has that class.</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>CL_MMA_ROLLUP MED_CLASS</t>
+          <t>CL_MMA_ROLLUP</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Mirror LOT1 dynamic class flag generation. STEROID class excluded.</t>
+          <t>Mirror LOT1 dynamic class flag generation.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr"/>
@@ -1572,7 +1556,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Flag: any valid AUTO SCT during LOT N</t>
+          <t>Any valid AUTO SCT during LOT N</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -1582,17 +1566,17 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Binary flag indicating the patient received any valid autologous SCT during LOT N (single or tandem).</t>
+          <t>Patient had &gt;=1 valid AUTO during LOT N.</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>CL_SCT_CODELIST (SCT_TYPE='AUTO')</t>
+          <t>CL_SCT_CODELIST (AUTO)</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Same logic as LOT1: 14-day windowing of T_MEDICAL procedure code dates; 60-day gap validation between distinct events.</t>
+          <t>Inherit LOT1 SCT logic: 14-day windowing, 60-day gap validation.</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr"/>
@@ -1610,7 +1594,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Flag: single valid AUTO SCT during LOT N</t>
+          <t>Single (non-tandem) AUTO during LOT N</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -1620,7 +1604,7 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Single AUTO not part of a valid tandem pair within LOT N.</t>
+          <t>AUTO not part of a valid tandem pair.</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -1628,11 +1612,7 @@
           <t>CL_SCT_CODELIST</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>Inherits LOT1 SCT logic.</t>
-        </is>
-      </c>
+      <c r="G11" s="7" t="inlineStr"/>
       <c r="H11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
@@ -1648,7 +1628,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Flag: planned tandem AUTO SCT during LOT N</t>
+          <t>Planned tandem AUTO during LOT N</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -1658,7 +1638,7 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Two AUTO SCTs within LOT N that are &gt;=60 and &lt;=180 days apart (planned tandem).</t>
+          <t>Two AUTOs &gt;=60 and &lt;=180 days apart.</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -1668,7 +1648,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Use datediff(AUTO_DT_2, AUTO_DT_1) without +1 (per Apr 22 protocol resolution).</t>
+          <t>Use datediff without +1 (per Apr 22).</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr"/>
@@ -1686,7 +1666,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Dates of first/second valid AUTO during LOT N</t>
+          <t>First / second valid AUTO date in LOT N</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -1696,7 +1676,7 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>AUTO_DT_1 is the first valid AUTO SCT during LOT N; AUTO_DT_2 is the second when a planned tandem exists.</t>
+          <t>DT_2 populated only if planned tandem.</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -1704,11 +1684,7 @@
           <t>CL_SCT_CODELIST</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>14-day windowing groups same-event claims; 60-day gap validates distinct events.</t>
-        </is>
-      </c>
+      <c r="G13" s="7" t="inlineStr"/>
       <c r="H13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
@@ -1724,7 +1700,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Latest valid AUTO SCT date during LOT N</t>
+          <t>Latest valid AUTO in LOT N</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -1734,7 +1710,7 @@
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Date of AUTO_DT_2 if a valid tandem; else AUTO_DT_1 if a single AUTO occurred; else NULL.</t>
+          <t>AUTO_DT_2 if tandem else AUTO_DT_1 else NULL.</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
@@ -1758,27 +1734,26 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Flag: LOT N regimen contains valid maintenance subset</t>
+          <t>LOT N regimen contains valid maintenance subset</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>0 / 1</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>Set 1 when LOT N induction regimen contains BOTH (a) at least one valid mono-maintenance agent OR a valid dual-maintenance combination, AND (b) at least one additional non-maintenance anchor agent. Same definition as LOT1. Valid mono: lenalidomide, bortezomib, daratumumab, ixazomib, thalidomide. Valid dual: bortezomib/lenalidomide, carfilzomib/lenalidomide, daratumumab/lenalidomide.</t>
-        </is>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="E15" s="7">
+        <f> 1 when LOT N induction has BOTH (a) &gt;=1 valid mono-maintenance agent OR a valid dual combo, AND (b) a non-maintenance anchor. Mono: LENA, BORT, DARA, IXAZ, THAL. Dual: BORT+LENA, CARF+LENA, DARA+LENA.</f>
+        <v/>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>CL_MMA_ROLLUP MONOMAINTENANCE / DUALMAINTENANCEWITH</t>
+          <t>CL_MMA_ROLLUP</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Descriptive flag only; does NOT derive a separate maintenance LOT or maintenance end date.</t>
+          <t>Descriptive flag; no standalone maintenance LOT.</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr"/>
@@ -1796,7 +1771,7 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Flag: LOT N is an allogeneic SCT line</t>
+          <t>LOT N is an ALLO SCT line</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -1804,21 +1779,16 @@
           <t>0/1</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>Set 1 when LOTN_START_TYPE='SCT_ALLO'. Per protocol: an allogeneic SCT is classified as its own LOT, with no other MM therapies included in that LOT. LOT span is the ALLO date itself (start = end = ALLO date) unless followed by a regimen that initiates LOT_(N+1).</t>
-        </is>
+      <c r="E16" s="7">
+        <f> 1 when LOTN_START_TYPE = SCT_ALLO. ALLO LOT contains no MM therapies. Span: see Q2 (draft = single day).</f>
+        <v/>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>CL_SCT_CODELIST (SCT_TYPE='ALLO')</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr">
-        <is>
-          <t>Open question: should LOTN_BASE_END_DT be the ALLO date (one-day LOT) or extend to the day before LOT_(N+1) start? See Open_Questions tab Q2.</t>
-        </is>
-      </c>
+          <t>CL_SCT_CODELIST (ALLO)</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr"/>
       <c r="H16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1834,7 +1804,7 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Flag: LOT N is a CAR-T line</t>
+          <t>LOT N is a CAR-T line</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -1842,19 +1812,18 @@
           <t>0/1</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>Set 1 when LOTN_START_TYPE='CART'. CAR-T is its own LOT; oncology agents (incl. supportive, e.g., corticosteroids) given within 45 days of CAR-T are CONSOLIDATED into the CAR-T LOT and not treated as new induction. PROVENANCE: 45-day consolidation per Apr 22 study-team decision (supersedes 30-day older protocol text); see Q11.</t>
-        </is>
+      <c r="E17" s="7">
+        <f> 1 when LOTN_START_TYPE = CART. Agents within 45d of FIRST_CART_DT are consolidated into LOT N (Apr 22 decision; see Q11).</f>
+        <v/>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>CL_SCT_CODELIST (SCT_TYPE='CART')</t>
+          <t>CL_SCT_CODELIST (CART)</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Within 45-day consolidation window, do NOT advance to LOT_(N+1). Use FIRST_CART_DT as LOTN_START_DT.</t>
+          <t>Do NOT advance to LOT_(N+1) for consolidated agents.</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr"/>
@@ -1869,8 +1838,7 @@
     <row r="21" ht="60" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Example A - LOT2 starts on a NEW MEDICATION (most common case).
-Patient was on VRd (bortezomib + lenalidomide + dexamethasone) for LOT1. LOT1 ended on 2025-08-19 with reason MED_ADD because daratumumab was added on 2025-08-20. The patient receives DARA on 2025-08-20 and lenalidomide refills appear within 30 days. No SCT or CAR-T occurs.</t>
+          <t>VRd in LOT1; DARA added 2025-08-20 (LOT1 ends 2025-08-19, MED_ADD). LENA refills present within 30d. No SCT/CAR-T.</t>
         </is>
       </c>
       <c r="B21" s="10" t="n"/>
@@ -2177,8 +2145,7 @@
     <row r="38" ht="60" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>Example B - LOT2 starts on an ALLOGENEIC SCT.
-Patient on VRd in LOT1 receives an allogeneic SCT on 2025-09-15. Per protocol, ALLO is its own LOT with no other MM therapies. LOT1 ends 2025-09-14 (day before ALLO). Next MM therapy after the ALLO date is daratumumab on 2025-12-10, which starts LOT3.</t>
+          <t>VRd in LOT1; ALLO on 2025-09-15 (LOT1 ends 2025-09-14). Next MM therapy DARA on 2025-12-10 starts LOT3.</t>
         </is>
       </c>
       <c r="B38" s="10" t="n"/>
@@ -2385,8 +2352,7 @@
     <row r="51" ht="60" customHeight="1">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>Example C - LOT2 starts on an UNPLANNED autologous SCT.
-Patient had a single AUTO during LOT1 on 2025-03-01. A second AUTO occurs on 2025-10-15 - 228 days later, which is &gt;180 days, so it is unplanned. The unplanned AUTO ends LOT1 (2025-10-14) and starts LOT2 on the AUTO date itself.</t>
+          <t>Single AUTO 2025-03-01 in LOT1; second AUTO 2025-10-15 (228d later, unplanned). LOT1 ends 2025-10-14; LOT2 starts on AUTO.</t>
         </is>
       </c>
       <c r="B51" s="10" t="n"/>
@@ -2614,7 +2580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2682,7 +2648,7 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Temporary end date for LOT N base period</t>
+          <t>Temporary LOT N end date</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
@@ -2692,17 +2658,17 @@
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>PRIMARY analysis - LOT N continues until the earliest of: (1) Discontinuation of all agents in the regimen (with or without switch to a new agent) - end date is the run-out date (last MAP_END_DT among induction agents); (2) Addition of a qualifying new MM oncology agent not in the LOT N induction regimen and not a permissible biosimilar substitute - end date is the day before the new agent's MAP_START_DT; (3) SCT/CAR-T events: any ALLO SCT ends the LOT the day before the ALLO; an AUTO SCT &gt;180 days after a previous AUTO ends LOT the day before; CAR-T infusion ends the LOT the day before FIRST_CART_DT; (4) Death (T_DOD.YMDOD); (5) End of the study period (study_end config). Health plan disenrollment is NOT a primary LOT-ending event. SENSITIVITY analysis - when CENSOR_AT_DISENROLLMENT = TRUE, LOT N observation end is additionally capped at ENDDATE_CE (see LOTN_END_REASON_CE_SENS below).</t>
+          <t>PRIMARY: earliest of (1) all-agent discontinuation (run-out date); (2) new qualifying MM agent (day before MAP_START_DT); (3) ALLO SCT (day before); (4) unplanned AUTO &gt;180d after prior AUTO (day before); (5) CAR-T (day before FIRST_CART_DT); (6) death (YMDOD); (7) study_end. Disenrollment is NOT a primary end event. SENSITIVITY: additionally cap at ENDDATE_CE when CENSOR_AT_DISENROLLMENT = TRUE.</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>T_MEDICAL/T_RX (MAP_END_DT, MAP_START_DT), T_MEDICAL procedure codes (SCT/CAR-T), T_DOD (YMDOD), study_end config; SENSITIVITY only: T_MEMBER_CONT_ENROLLMENT (ELIGEND -&gt; ENDDATE_CE)</t>
+          <t>T_MEDICAL/T_RX, T_DOD, study_end; SENSITIVITY: T_MEMBER_CONT_ENROLLMENT (ELIGEND)</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
-          <t>Primary path mirrors current LOT1 implementation: ignores disenrollment. Same priority logic as LOT1; only the induction window differs.</t>
+          <t>Primary path inherits LOT1 logic; only induction window differs.</t>
         </is>
       </c>
       <c r="H2" s="7" t="inlineStr"/>
@@ -2720,7 +2686,7 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>LOT N discontinuation date</t>
+          <t>LOT N run-out date</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
@@ -2730,7 +2696,7 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Run-out date: max(MAP_END_DT) across LOT N induction medications. If regimen is discontinued and no new agent is initiated, LOT end date is this run-out date. If interrupted by a new agent on or before the run-out date, LOT end is day before the new agent.</t>
+          <t>max(MAP_END_DT) across LOT N induction agents. Used as LOT end when reason = DISCONTINUATION.</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -2740,7 +2706,7 @@
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>Source: T_MEDICAL (FST_DT + medical_day_supply - 1), T_RX (FILL_DT + DAYS_SUP - 1) for induction meds. Pharmacy claims with missing/anomalous DAY_SUPPLY use 28-day default (per protocol; see C2 of Apr 15 review).</t>
+          <t>T_MEDICAL: FST_DT + medical_day_supply - 1. T_RX: FILL_DT + DAYS_SUP - 1. Missing DAY_SUPPLY -&gt; 28d default (do not delete claims).</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr"/>
@@ -2758,7 +2724,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Date and name of first non-induction medication added during LOT N</t>
+          <t>First non-induction agent during LOT N</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -2768,17 +2734,17 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>First MM oncology agent (non-steroid) appearing AFTER the induction window with MAP_START_DT on or before LOTN_BASE_DISCON_DT, and not already part of LOTN_BASE_MEDS or its permissible biosimilar substitute.</t>
+          <t>First non-steroid MM agent after the induction window with MAP_START_DT &lt;= LOTN_BASE_DISCON_DT, not in LOTN_BASE_MEDS or its biosimilar.</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>CL_MMA_CODELIST, CL_MMA_ROLLUP, permissible_subs</t>
+          <t>CL_MMA_CODELIST, permissible_subs</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>Filter MAP_MED_CLASS != 'STEROID'. Validate against permissible_subs reference table before classifying as new add.</t>
+          <t>Check permissible_subs before classifying as new add.</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr"/>
@@ -2796,7 +2762,7 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Discontinuation gap threshold (days)</t>
+          <t>Discontinuation gap (days)</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -2806,7 +2772,7 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Inherits LOT1 protocol value: discontinuation = all MM agents in LOT have stopped (run-out reached) and no new agent within gap.</t>
+          <t>Inherits LOT1.</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -2814,11 +2780,7 @@
           <t>n/a</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>Same as LOT1; sensitivity analyses may vary 30/60/90.</t>
-        </is>
-      </c>
+      <c r="G5" s="7" t="inlineStr"/>
       <c r="H5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
@@ -2834,7 +2796,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Assumed days supply for medical claims</t>
+          <t>Assumed medical days supply</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -2844,7 +2806,7 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Medical-claim days supply is missing; assume 28 days. Pharmacy claims with missing or anomalous days supply also default to 28.</t>
+          <t>Default for missing/anomalous DAY_SUPPLY (medical and pharmacy).</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -2854,7 +2816,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Apply COALESCE/CASE; do NOT delete claims with missing DAY_SUPPLY.</t>
+          <t>Use COALESCE; do NOT delete claims.</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr"/>
@@ -2872,7 +2834,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Allogeneic SCT always ends current LOT</t>
+          <t>ALLO always ends current LOT</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -2882,19 +2844,15 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Any ALLO SCT immediately ends the current LOT (day before the ALLO) and begins a new LOT (the ALLO LOT).</t>
+          <t>Any ALLO ends current LOT day before ALLO, and starts a new ALLO LOT.</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>CL_SCT_CODELIST (SCT_TYPE='ALLO')</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>Same as LOT1.</t>
-        </is>
-      </c>
+          <t>CL_SCT_CODELIST (ALLO)</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr"/>
       <c r="H7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
@@ -2910,7 +2868,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Tandem AUTO classification window</t>
+          <t>Tandem AUTO window</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -2920,17 +2878,17 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Two AUTO SCTs &gt;=60 and &lt;=180 days apart are planned tandem (continuation of same LOT). &gt;180 days apart triggers a new LOT.</t>
+          <t>Two AUTOs &gt;=60 and &lt;=180 days apart = planned tandem (same LOT). &gt;180 days = unplanned (new LOT).</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>CL_SCT_CODELIST (SCT_TYPE='AUTO')</t>
+          <t>CL_SCT_CODELIST (AUTO)</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Use datediff without +1 (per Apr 22 resolution).</t>
+          <t>Use datediff without +1.</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr"/>
@@ -2948,7 +2906,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>CAR-T consolidation window (days)</t>
+          <t>CAR-T consolidation window</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -2958,17 +2916,17 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Oncology therapies (including supportive agents like steroids) given within 45 days of FIRST_CART_DT are consolidated into the CAR-T LOT. PROVENANCE: per Apr 22, 2026 study-team decision, the CAR-T consolidation window is 45 days. This supersedes the earlier 30-day language in the protocol extract; treat 45 as the operative value for LOT2-5 (matches LOT1 CART_INIT).</t>
+          <t>Agents within 45d of FIRST_CART_DT are consolidated into the CAR-T LOT. Apr 22 study-team decision (Q11).</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>CL_SCT_CODELIST (SCT_TYPE='CART')</t>
+          <t>CL_SCT_CODELIST (CART)</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Reclassify therapies within 45-day window into the CAR-T LOT; do NOT trigger LOT_(N+1) for those agents.</t>
+          <t>Do NOT advance to LOT_(N+1) for consolidated agents.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr"/>
@@ -2986,7 +2944,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Final LOT N base period end date</t>
+          <t>Final LOT N end date (PRIMARY)</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -2996,17 +2954,17 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Earliest of all qualifying end events. For ALLO/CAR-T-started LOTs (LOTN_START_TYPE in ('SCT_ALLO','CART')), see special handling in Open_Questions tab Q2.</t>
+          <t>Earliest qualifying end event from LOTN_END_DT_TEMP.</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>All sources above</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Priority logic same as LOT1.</t>
+          <t>ALLO/CAR-T LOT span: see Q2.</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr"/>
@@ -3024,7 +2982,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Final LOT N base end reason (PRIMARY analysis)</t>
+          <t>Final LOT N end reason (PRIMARY)</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -3034,17 +2992,17 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Final reason for the PRIMARY analysis. Priority when ties on the same day: SCT_ALLO &gt; SCT_CART &gt; SCT_AUTO &gt; CART_INIT &gt; MED_ADD &gt; DISCONTINUATION &gt; DEATH &gt; STUDY_END. DISENROLLMENT is NOT a primary end reason - it appears only in the sensitivity output (LOTN_BASE_END_REASON_CE_SENS).</t>
+          <t>Reason corresponding to LOTN_BASE_END_DT. DISENROLLMENT only in sensitivity (see *_CE_SENS).</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>All sources above (excluding T_MEMBER_CONT_ENROLLMENT for primary)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Same priority order as LOT1. CART_INIT applies when CAR-T occurs within 45 days of a first added agent during LOT N.</t>
+          <t>DRAFT same-day priority (inherits LOT1 - confirm): SCT_ALLO &gt; SCT_CART &gt; SCT_AUTO &gt; CART_INIT &gt; MED_ADD &gt; DISCONTINUATION &gt; DEATH &gt; STUDY_END. CART_INIT logic inherits LOT1 (CAR-T within 45d of first add) - confirm applies to LOT2-5.</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr"/>
@@ -3062,7 +3020,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>LOT N base end date - sensitivity (censor at disenrollment)</t>
+          <t>LOT N end date (SENSITIVITY)</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -3072,17 +3030,17 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Sensitivity-analysis end date computed identically to LOTN_BASE_END_DT but additionally capped at ENDDATE_CE = min(YMDOD, ELIGEND, study_end). Only emitted when CENSOR_AT_DISENROLLMENT = TRUE.</t>
+          <t>Same as LOTN_BASE_END_DT, additionally capped at ELIGEND. Emitted when CENSOR_AT_DISENROLLMENT = TRUE.</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>T_MEMBER_CONT_ENROLLMENT (ELIGEND), T_DOD, study_end config</t>
+          <t>T_MEMBER_CONT_ENROLLMENT</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Sensitivity flag-gated; primary LOTN_BASE_END_DT remains untouched.</t>
+          <t>Primary LOTN_BASE_END_DT untouched.</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr"/>
@@ -3100,27 +3058,27 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>LOT N base end reason - sensitivity</t>
+          <t>LOT N end reason (SENSITIVITY)</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>SCT_ALLO / SCT_CART / SCT_AUTO / CART_INIT / MED_ADD / DISCONTINUATION / DEATH / DISENROLLMENT / STUDY_END</t>
+          <t>(primary set) + DISENROLLMENT</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Final reason for the sensitivity analysis. DISENROLLMENT is emitted when ELIGEND is the binding earliest cap. Priority order extends the primary list: SCT_ALLO &gt; SCT_CART &gt; SCT_AUTO &gt; CART_INIT &gt; MED_ADD &gt; DISCONTINUATION &gt; DEATH &gt; DISENROLLMENT &gt; STUDY_END.</t>
+          <t>Same as primary, plus DISENROLLMENT when ELIGEND binds.</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>All sources above plus T_MEMBER_CONT_ENROLLMENT (ELIGEND)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>REQUIRED behaviour: when sensitivity ENDDATE_CE binds because of disenrollment (ELIGEND earliest), label the reason DISENROLLMENT (do NOT collapse to STUDY_END). This is a deliberate divergence from the current LOT1 implementation, which labels the cap as STUDY_END; LOT2-5 should emit DISENROLLMENT for analytic clarity.</t>
+          <t>REQUIRED: emit DISENROLLMENT (do NOT collapse to STUDY_END). Diverges from current LOT1 behaviour.</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr"/>
@@ -3138,7 +3096,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>LOT N base period duration in days</t>
+          <t>LOT N duration (days)</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -3148,7 +3106,7 @@
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>If LOTN_BASE_END_REASON = 'DISCONTINUATION' then LOTN_BASE_DISCON_DT - LOTN_START_DT + 1; else LOTN_BASE_END_DT - LOTN_START_DT + 1.</t>
+          <t>If reason = DISCONTINUATION: LOTN_BASE_DISCON_DT - LOTN_START_DT + 1. Else: LOTN_BASE_END_DT - LOTN_START_DT + 1.</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
@@ -3158,7 +3116,7 @@
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Confirm censored-patient handling against LOT1 M1 finding (Apr 15 review).</t>
+          <t>Confirm censored handling (LOT1 M1).</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr"/>
@@ -3176,7 +3134,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Permissible biosimilar substitution rules</t>
+          <t>Biosimilar substitution rule</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -3186,19 +3144,15 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Substitution of a biologic reference product with any of its biosimilars, or between biosimilars of the same reference product, does not advance the LOT. The LOT is named by the drug given for the longest duration.</t>
+          <t>Biosimilar swap within a reference product family does not end/advance the LOT. Regimen named by longest-duration drug.</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>permissible_subs reference</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>Same as LOT1.</t>
-        </is>
-      </c>
+          <t>permissible_subs</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr"/>
       <c r="H15" s="7" t="inlineStr"/>
     </row>
     <row r="18" ht="22" customHeight="1">
@@ -3211,13 +3165,7 @@
     <row r="19" ht="60" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>Example D - END-REASON RESOLUTION (priority logic).
-LOT3 started 2025-11-01 with KRd. The patient has multiple competing end events:
-  - Run-out date of induction agents (DISCONTINUATION candidate): 2026-04-15
-  - First add med (POMA) on 2026-03-20 -&gt; LOT3 would end 2026-03-19 (MED_ADD)
-  - CAR-T infusion on 2026-04-02 (within 45 days of POMA)  -&gt; CART_INIT applies
-  - Death (YMDOD) on 2026-05-20
-Apply priority: SCT_ALLO &gt; SCT_CART &gt; SCT_AUTO &gt; CART_INIT &gt; MED_ADD &gt; DISCONTINUATION &gt; DEATH &gt; STUDY_END.</t>
+          <t>LOT3 starts 2025-11-01 (KRd). Competing events: run-out 2026-04-15; POMA add 2026-03-20; CAR-T 2026-04-02 (within 45d of POMA); death 2026-05-20. Priority resolves to CART_INIT.</t>
         </is>
       </c>
       <c r="B19" s="10" t="n"/>
@@ -3263,7 +3211,7 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>FIRST_CART_DT (2026-04-02) - 1. CART_INIT outranks MED_ADD because CAR-T occurred within 45d of the first add.</t>
+          <t>FIRST_CART_DT - 1.</t>
         </is>
       </c>
       <c r="D21" s="9" t="n"/>
@@ -3285,7 +3233,7 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Highest-priority qualifying reason among competing events.</t>
+          <t>CART_INIT outranks MED_ADD; CAR-T within 45d of first add.</t>
         </is>
       </c>
       <c r="D22" s="9" t="n"/>
@@ -3307,7 +3255,7 @@
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>2026-04-01 minus 2025-11-01 + 1 = 152 days.</t>
+          <t>2026-04-01 - 2025-11-01 + 1.</t>
         </is>
       </c>
       <c r="D23" s="9" t="n"/>
@@ -3329,7 +3277,7 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>FIRST_CART_DT becomes LOT4 start; LOT4_START_TYPE = CART.</t>
+          <t>LOT4_START_TYPE = CART.</t>
         </is>
       </c>
       <c r="D24" s="9" t="n"/>
@@ -3338,104 +3286,107 @@
       <c r="G24" s="9" t="n"/>
       <c r="H24" s="9" t="n"/>
     </row>
-    <row r="25">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t>LOTN_BASE_END_DT_CE_SENS</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>Same as primary - no disenrollment cap binds earlier.</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="9" t="n"/>
-      <c r="F25" s="9" t="n"/>
-      <c r="G25" s="9" t="n"/>
-      <c r="H25" s="9" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="13" t="inlineStr">
-        <is>
-          <t>LOTN_BASE_END_REASON_CE_SENS</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>CART_INIT</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr"/>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="9" t="n"/>
-      <c r="F26" s="9" t="n"/>
-      <c r="G26" s="9" t="n"/>
-      <c r="H26" s="9" t="n"/>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="8" t="inlineStr">
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>WORKED EXAMPLE E - Discontinuation (run-out)</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="60" customHeight="1">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>Example E - DISCONTINUATION (regimen runs out, no new agent within gap).
-LOT2 started 2025-08-20 with DARA + LENA. Last LENA fill (28-day supply) is 2026-01-10, MAP_END_DT = 2026-02-06. Last DARA infusion MAP_END_DT = 2026-01-15. No new MM agent appears in the next 90 days. Patient is alive and enrolled.</t>
-        </is>
-      </c>
-      <c r="B30" s="10" t="n"/>
-      <c r="C30" s="10" t="n"/>
-      <c r="D30" s="10" t="n"/>
-      <c r="E30" s="10" t="n"/>
-      <c r="F30" s="10" t="n"/>
-      <c r="G30" s="10" t="n"/>
-      <c r="H30" s="11" t="n"/>
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>LOT2 starts 2025-08-20 (DARA+LENA). Last LENA MAP_END_DT 2026-02-06; last DARA 2026-01-15. No new agent in 90d.</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="10" t="n"/>
+      <c r="D28" s="10" t="n"/>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="10" t="n"/>
+      <c r="G28" s="10" t="n"/>
+      <c r="H28" s="11" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>Value for this patient</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>How it was derived</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="n"/>
+      <c r="E29" s="12" t="n"/>
+      <c r="F29" s="12" t="n"/>
+      <c r="G29" s="12" t="n"/>
+      <c r="H29" s="12" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_DISCON_DT</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>max(MAP_END_DT) across LOT2 induction agents.</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="n"/>
+      <c r="E30" s="9" t="n"/>
+      <c r="F30" s="9" t="n"/>
+      <c r="G30" s="9" t="n"/>
+      <c r="H30" s="9" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
-      </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>Value for this patient</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>How it was derived</t>
-        </is>
-      </c>
-      <c r="D31" s="12" t="n"/>
-      <c r="E31" s="12" t="n"/>
-      <c r="F31" s="12" t="n"/>
-      <c r="G31" s="12" t="n"/>
-      <c r="H31" s="12" t="n"/>
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_END_DT</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>Run-out date itself when reason = DISCONTINUATION.</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="n"/>
+      <c r="E31" s="9" t="n"/>
+      <c r="F31" s="9" t="n"/>
+      <c r="G31" s="9" t="n"/>
+      <c r="H31" s="9" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>LOTN_BASE_DISCON_DT</t>
+          <t>LOTN_BASE_END_REASON</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>DISCONTINUATION</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>max(MAP_END_DT) across LOT2 induction agents (the later LENA run-out).</t>
+          <t>Run-out reached; no agent within 90d gap.</t>
         </is>
       </c>
       <c r="D32" s="9" t="n"/>
@@ -3447,17 +3398,17 @@
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>LOTN_BASE_END_DT</t>
+          <t>LOTN_BASE_LENGTH</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>171</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>DISCONTINUATION uses the run-out date itself.</t>
+          <t>2026-02-06 - 2025-08-20 + 1.</t>
         </is>
       </c>
       <c r="D33" s="9" t="n"/>
@@ -3466,130 +3417,125 @@
       <c r="G33" s="9" t="n"/>
       <c r="H33" s="9" t="n"/>
     </row>
-    <row r="34">
-      <c r="A34" s="13" t="inlineStr">
-        <is>
-          <t>LOTN_BASE_END_REASON</t>
-        </is>
-      </c>
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t>DISCONTINUATION</t>
-        </is>
-      </c>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t>All agents reached run-out and no new agent within 90-day gap.</t>
-        </is>
-      </c>
-      <c r="D34" s="9" t="n"/>
-      <c r="E34" s="9" t="n"/>
-      <c r="F34" s="9" t="n"/>
-      <c r="G34" s="9" t="n"/>
-      <c r="H34" s="9" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="13" t="inlineStr">
-        <is>
-          <t>LOTN_BASE_LENGTH</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>171</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>2026-02-06 minus 2025-08-20 + 1.</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="n"/>
-      <c r="E35" s="9" t="n"/>
-      <c r="F35" s="9" t="n"/>
-      <c r="G35" s="9" t="n"/>
-      <c r="H35" s="9" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="13" t="inlineStr">
-        <is>
-          <t>Next LOT?</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t>Only if a new MM agent eventually appears</t>
-        </is>
-      </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>If no further therapy, study/death/sensitivity will eventually close follow-up.</t>
-        </is>
-      </c>
-      <c r="D36" s="9" t="n"/>
-      <c r="E36" s="9" t="n"/>
-      <c r="F36" s="9" t="n"/>
-      <c r="G36" s="9" t="n"/>
-      <c r="H36" s="9" t="n"/>
-    </row>
-    <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="8" t="inlineStr">
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>WORKED EXAMPLE F - Disenrollment primary vs sensitivity</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="60" customHeight="1">
-      <c r="A40" s="9" t="inlineStr">
-        <is>
-          <t>Example F - DISENROLLMENT: primary analysis vs sensitivity analysis.
-LOT4 started 2026-01-05. Patient disenrolls (ELIGEND) on 2026-04-30 with no death and no further therapy. study_end is 2026-12-31. This shows how the same patient produces different LOT4 closures under primary vs sensitivity.</t>
-        </is>
-      </c>
-      <c r="B40" s="10" t="n"/>
-      <c r="C40" s="10" t="n"/>
-      <c r="D40" s="10" t="n"/>
-      <c r="E40" s="10" t="n"/>
-      <c r="F40" s="10" t="n"/>
-      <c r="G40" s="10" t="n"/>
-      <c r="H40" s="11" t="n"/>
+    <row r="37" ht="60" customHeight="1">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>LOT4 starts 2026-01-05. ELIGEND 2026-04-30; no death; study_end 2026-12-31.</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="n"/>
+      <c r="C37" s="10" t="n"/>
+      <c r="D37" s="10" t="n"/>
+      <c r="E37" s="10" t="n"/>
+      <c r="F37" s="10" t="n"/>
+      <c r="G37" s="10" t="n"/>
+      <c r="H37" s="11" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>Value for this patient</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>How it was derived</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="n"/>
+      <c r="E38" s="12" t="n"/>
+      <c r="F38" s="12" t="n"/>
+      <c r="G38" s="12" t="n"/>
+      <c r="H38" s="12" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_END_DT (PRIMARY)</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>Disenrollment ignored; min(death, study_end) = study_end.</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="n"/>
+      <c r="E39" s="9" t="n"/>
+      <c r="F39" s="9" t="n"/>
+      <c r="G39" s="9" t="n"/>
+      <c r="H39" s="9" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_END_REASON (PRIMARY)</t>
+        </is>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>STUDY_END</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr"/>
+      <c r="D40" s="9" t="n"/>
+      <c r="E40" s="9" t="n"/>
+      <c r="F40" s="9" t="n"/>
+      <c r="G40" s="9" t="n"/>
+      <c r="H40" s="9" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="12" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
-      </c>
-      <c r="B41" s="12" t="inlineStr">
-        <is>
-          <t>Value for this patient</t>
-        </is>
-      </c>
-      <c r="C41" s="12" t="inlineStr">
-        <is>
-          <t>How it was derived</t>
-        </is>
-      </c>
-      <c r="D41" s="12" t="n"/>
-      <c r="E41" s="12" t="n"/>
-      <c r="F41" s="12" t="n"/>
-      <c r="G41" s="12" t="n"/>
-      <c r="H41" s="12" t="n"/>
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_END_DT_CE_SENS</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>ELIGEND binds.</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="n"/>
+      <c r="E41" s="9" t="n"/>
+      <c r="F41" s="9" t="n"/>
+      <c r="G41" s="9" t="n"/>
+      <c r="H41" s="9" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>LOTN_BASE_END_DT (PRIMARY)</t>
+          <t>LOTN_BASE_END_REASON_CE_SENS</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>2026-12-31</t>
+          <t>DISENROLLMENT</t>
         </is>
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Disenrollment is IGNORED in primary; earliest of {death, study_end} = study_end.</t>
+          <t>Required: do NOT collapse to STUDY_END.</t>
         </is>
       </c>
       <c r="D42" s="9" t="n"/>
@@ -3601,17 +3547,17 @@
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>LOTN_BASE_END_REASON (PRIMARY)</t>
+          <t>LOTN_BASE_LENGTH (PRIMARY)</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>STUDY_END</t>
+          <t>361</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>Primary analysis cannot use DISENROLLMENT.</t>
+          <t>2026-12-31 - 2026-01-05 + 1.</t>
         </is>
       </c>
       <c r="D43" s="9" t="n"/>
@@ -3623,17 +3569,17 @@
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>LOTN_BASE_END_DT_CE_SENS (SENSITIVITY)</t>
+          <t>LOTN_BASE_LENGTH_CE_SENS</t>
         </is>
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>116</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>ENDDATE_CE = min(YMDOD, ELIGEND, study_end) = ELIGEND.</t>
+          <t>2026-04-30 - 2026-01-05 + 1.</t>
         </is>
       </c>
       <c r="D44" s="9" t="n"/>
@@ -3642,100 +3588,31 @@
       <c r="G44" s="9" t="n"/>
       <c r="H44" s="9" t="n"/>
     </row>
-    <row r="45">
-      <c r="A45" s="13" t="inlineStr">
-        <is>
-          <t>LOTN_BASE_END_REASON_CE_SENS (SENSITIVITY)</t>
-        </is>
-      </c>
-      <c r="B45" s="9" t="inlineStr">
-        <is>
-          <t>DISENROLLMENT</t>
-        </is>
-      </c>
-      <c r="C45" s="9" t="inlineStr">
-        <is>
-          <t>Spec requires labelling DISENROLLMENT (do NOT collapse to STUDY_END).</t>
-        </is>
-      </c>
-      <c r="D45" s="9" t="n"/>
-      <c r="E45" s="9" t="n"/>
-      <c r="F45" s="9" t="n"/>
-      <c r="G45" s="9" t="n"/>
-      <c r="H45" s="9" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="13" t="inlineStr">
-        <is>
-          <t>LOTN_BASE_LENGTH (PRIMARY)</t>
-        </is>
-      </c>
-      <c r="B46" s="9" t="inlineStr">
-        <is>
-          <t>361</t>
-        </is>
-      </c>
-      <c r="C46" s="9" t="inlineStr">
-        <is>
-          <t>2026-12-31 minus 2026-01-05 + 1.</t>
-        </is>
-      </c>
-      <c r="D46" s="9" t="n"/>
-      <c r="E46" s="9" t="n"/>
-      <c r="F46" s="9" t="n"/>
-      <c r="G46" s="9" t="n"/>
-      <c r="H46" s="9" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="13" t="inlineStr">
-        <is>
-          <t>LOTN_BASE_LENGTH_CE_SENS</t>
-        </is>
-      </c>
-      <c r="B47" s="9" t="inlineStr">
-        <is>
-          <t>116</t>
-        </is>
-      </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>2026-04-30 minus 2026-01-05 + 1.</t>
-        </is>
-      </c>
-      <c r="D47" s="9" t="n"/>
-      <c r="E47" s="9" t="n"/>
-      <c r="F47" s="9" t="n"/>
-      <c r="G47" s="9" t="n"/>
-      <c r="H47" s="9" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="26">
-    <mergeCell ref="C25:H25"/>
+  <mergeCells count="23">
     <mergeCell ref="C41:H41"/>
-    <mergeCell ref="A30:H30"/>
-    <mergeCell ref="A39:H39"/>
-    <mergeCell ref="C47:H47"/>
     <mergeCell ref="C44:H44"/>
     <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C40:H40"/>
     <mergeCell ref="C31:H31"/>
+    <mergeCell ref="A36:H36"/>
     <mergeCell ref="C43:H43"/>
     <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C46:H46"/>
-    <mergeCell ref="C36:H36"/>
     <mergeCell ref="C23:H23"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A27:H27"/>
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="C32:H32"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="C38:H38"/>
+    <mergeCell ref="C30:H30"/>
     <mergeCell ref="C33:H33"/>
     <mergeCell ref="C24:H24"/>
     <mergeCell ref="C42:H42"/>
-    <mergeCell ref="A29:H29"/>
-    <mergeCell ref="C45:H45"/>
+    <mergeCell ref="A28:H28"/>
     <mergeCell ref="A19:H19"/>
-    <mergeCell ref="C35:H35"/>
-    <mergeCell ref="C26:H26"/>
     <mergeCell ref="C20:H20"/>
+    <mergeCell ref="C29:H29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3750,12 +3627,12 @@
   <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3793,12 +3670,12 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>Allogeneic SCT (ALLO)</t>
+          <t>ALLO SCT</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Always - any ALLO ends the current LOT and starts a new ALLO LOT.</t>
+          <t>Always.</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
@@ -3808,7 +3685,7 @@
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>ALLO LOT contains NO MM therapies (per protocol). Subsequent MM therapy starts LOT_(N+1).</t>
+          <t>No MM therapies in this LOT.</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
@@ -3818,19 +3695,19 @@
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>Open question Q2: should this LOT be a single-day record (start=end=ALLO_DT) or extend until the next agent?</t>
+          <t>Q2: span = single day (draft).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>CAR-T infusion</t>
+          <t>CAR-T</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Always - CAR-T is its own LOT.</t>
+          <t>Always.</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
@@ -3840,39 +3717,39 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>Includes all oncology therapies (and supportive agents like steroids) within 45 days post-CAR-T (consolidation per Apr 22 decision).</t>
+          <t>Agents within 45d are consolidated into this LOT.</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>SCT_CART (or CART_INIT if CAR-T within 45d of a first-add agent in LOT_(N-1))</t>
+          <t>SCT_CART (or CART_INIT if CAR-T within 45d of first add in LOT_(N-1))</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Use 45-day consolidation window per Apr 22 study-team decision (supersedes 30-day protocol text).</t>
+          <t>45d per Apr 22 (Q11).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Autologous SCT (AUTO) - unplanned</t>
+          <t>Unplanned AUTO</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>AUTO occurs &gt;180 days after a previous AUTO in the same line. Competes as a first-class LOT-start trigger alongside MED, ALLO, CAR-T - whichever is earliest wins.</t>
+          <t>&gt;180d after prior AUTO in LOT_(N-1).</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>AUTO_DT (the latter, unplanned AUTO)</t>
+          <t>AUTO_DT</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Induction window 30 days from AUTO_DT.</t>
+          <t>30d induction from AUTO_DT.</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -3882,51 +3759,51 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>If within 60-180 days of prior AUTO, it is planned tandem and stays in the same LOT - does not start LOT_(N+1).</t>
+          <t>Planned tandem (60-180d) does NOT start a new LOT.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>New MM oncology agent</t>
+          <t>New MM agent</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>After LOT_(N-1) ends by DISCONTINUATION/MED_ADD with no SCT/CAR-T trigger.</t>
+          <t>After LOT_(N-1) ended by DISCONTINUATION or MED_ADD with no SCT/CAR-T.</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>MAP_START_DT of the first such agent post LOT_(N-1)_BASE_END_DT</t>
+          <t>MAP_START_DT of new agent</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>30-day induction window from LOTN_START_DT.</t>
+          <t>30d induction window.</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>n/a (this is the start of LOT N, not the end of LOT_(N-1))</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Steroids alone do not start a LOT. Permissible biosimilar substitutes do not start a LOT.</t>
+          <t>Steroids and biosimilar subs do not start a LOT.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Death / study end (PRIMARY)</t>
+          <t>Death / STUDY_END (PRIMARY)</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Never - these end follow-up; no LOT_(N+1).</t>
+          <t>Never starts a LOT; ends follow-up.</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -3946,19 +3823,19 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>LOT_(N-1) ends; no new LOT begins. Disenrollment is NOT a primary end event.</t>
+          <t>Disenrollment is NOT a primary end event.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Health plan disenrollment (SENSITIVITY ONLY)</t>
+          <t>Disenrollment (SENSITIVITY only)</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Never starts a new LOT. Sensitivity-only: when CENSOR_AT_DISENROLLMENT=TRUE, ELIGEND caps observation via ENDDATE_CE.</t>
+          <t>Never starts a LOT.</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -3973,12 +3850,12 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>DISENROLLMENT (sensitivity only; primary analysis ignores ELIGEND)</t>
+          <t>DISENROLLMENT (sensitivity)</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>PRIMARY analysis does NOT use disenrollment to end any LOT. SENSITIVITY emits LOTN_BASE_END_DT_CE_SENS / LOTN_BASE_END_REASON_CE_SENS only when the sensitivity flag is on. See Q12.</t>
+          <t>Cap via ENDDATE_CE only when CENSOR_AT_DISENROLLMENT = TRUE. Q12.</t>
         </is>
       </c>
     </row>
@@ -3996,9 +3873,9 @@
   <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -4021,85 +3898,85 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>S1. LOT1 ends by MED_ADD, LOT2 starts on new agent</t>
+          <t>S1. LOT1-&gt;LOT2 by MED_ADD</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Patient on VRd in LOT1; on day 200, daratumumab is added. LOT1 ends day 199 (MED_ADD); LOT2 starts day 200 with DARA.</t>
+          <t>VRd in LOT1; DARA added day 200.</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>LOT2_START_DT = day 200; LOT2_START_TYPE = MED. LOT2 induction window = day 200 to day 229 captures any agents started within 30 days. If only DARA appears in induction window -&gt; LOT2_BASE_MEDS = DARA.</t>
+          <t>LOT1 ends d199. LOT2_START_DT=d200, TYPE=MED. Induction d200-d229.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>S2. LOT1 ends by SCT_AUTO unplanned, LOT2 starts at AUTO date</t>
+          <t>S2. LOT1-&gt;LOT2 by unplanned AUTO</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Single AUTO SCT during LOT1 followed by another AUTO 220 days later. The second AUTO is unplanned (&gt;180d gap).</t>
+          <t>Single AUTO d100; second AUTO d320 (220d later).</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>LOT1 ends day before the second AUTO; LOT2_START_DT = second AUTO date; LOT2_START_TYPE = SCT_AUTO. LOT2 30-day induction captures any post-AUTO agents.</t>
+          <t>LOT1 ends d319. LOT2_START_DT=d320, TYPE=SCT_AUTO.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>S3. LOT1 ends by SCT_ALLO, LOT2 = ALLO LOT</t>
+          <t>S3. LOT1-&gt;LOT2 (ALLO LOT)-&gt;LOT3</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Patient receives ALLO during/after LOT1.</t>
+          <t>ALLO during/after LOT1, then later DARA.</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>LOT1 ends day before ALLO; LOT2_START_DT = ALLO_DT; LOT2_START_TYPE = SCT_ALLO; LOT2_ALLO_LOT_FLG = 1. LOT2 contains no MM therapies. Next MM agent starts LOT3.</t>
+          <t>LOT2: start=end=ALLO_DT (Q2 draft), no MM. Next agent starts LOT3.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>S4. LOT1 ends by CART, LOT2 = CAR-T LOT</t>
+          <t>S4. LOT1-&gt;LOT2 (CAR-T LOT)</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Patient receives CAR-T infusion.</t>
+          <t>CAR-T infusion.</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>LOT1 ends day before FIRST_CART_DT; LOT2_START_DT = FIRST_CART_DT; LOT2_START_TYPE = CART. Agents (incl. steroids) within 45 days post-CAR-T are part of LOT2. Next non-consolidated agent starts LOT3.</t>
+          <t>LOT2_START_DT=FIRST_CART_DT, TYPE=CART. Agents within 45d consolidated.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>S5. LOT2 -&gt; LOT3 by discontinuation then new agent</t>
+          <t>S5. LOT2-&gt;LOT3 by DISCONTINUATION</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>VRd in LOT2 ends by run-out (no new agent within 90d). Patient restarts therapy 200 days later with KRd.</t>
+          <t>Run-out, then new agent 200d later.</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>LOT2 ends on run-out (DISCONTINUATION). LOT3_START_DT = first KRd agent date; LOT3_START_TYPE = MED. 30-day induction captures K, R, d (steroid excluded from regimen).</t>
+          <t>LOT2 ends DISCONTINUATION. LOT3_START_DT = first new agent.</t>
         </is>
       </c>
     </row>
@@ -4111,97 +3988,97 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Patient dies during LOT3.</t>
+          <t>Death during LOT3.</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>LOT3_BASE_END_DT = YMDOD; LOT3_BASE_END_REASON = DEATH. No LOT4.</t>
+          <t>LOT3_BASE_END_DT=YMDOD, reason=DEATH. No LOT4.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>S6b. Disenrollment during LOT3 (primary vs sensitivity)</t>
+          <t>S6b. Disenrollment (primary vs sensitivity)</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Patient disenrolls (ELIGEND) during LOT3 with no death and no further therapy. Study end is later.</t>
+          <t>ELIGEND during LOT3, no death, study_end later.</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>PRIMARY: disenrollment is ignored. LOT3_BASE_END_REASON = STUDY_END (earliest of death/study_end), LOT3_BASE_END_DT = study_end. SENSITIVITY (CENSOR_AT_DISENROLLMENT=TRUE): LOT3_BASE_END_DT_CE_SENS = ELIGEND; LOT3_BASE_END_REASON_CE_SENS = DISENROLLMENT.</t>
+          <t>PRIMARY: reason=STUDY_END at study_end. SENSITIVITY: *_CE_SENS at ELIGEND, reason=DISENROLLMENT.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>S7. Tandem AUTO during LOT2</t>
+          <t>S7. Tandem AUTO in LOT2</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Two AUTO SCTs 90 days apart during LOT2.</t>
+          <t>Two AUTOs 90d apart.</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Both are planned tandem; LOT2 continues. LOT2_TX_AUTO_TAND_FLG = 1; LOT2_TX_AUTO_DT_1/DT_2 populated. LOT2 does not end on the second AUTO.</t>
+          <t>Planned tandem; LOT2 continues. AUTO_TAND_FLG=1.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>S8. Permissible biosimilar swap mid-LOT2</t>
+          <t>S8. Biosimilar swap in LOT2</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Patient on DARA in LOT2 switches to a DARA biosimilar.</t>
+          <t>DARA -&gt; DARA biosimilar.</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Substitution does NOT advance the LOT. LOT2 continues; regimen named by drug with longest duration.</t>
+          <t>LOT does not advance.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>S9. LOT2 base length = 1 day (ALLO LOT, open question)</t>
+          <t>S9. ALLO LOT span</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>ALLO is its own LOT; if no further therapy, what is LOT span?</t>
+          <t>ALLO with no follow-on therapy.</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Open question Q2. Draft assumption: LOT2_BASE_END_DT = ALLO_DT (1-day LOT); subsequent agents -&gt; LOT3.</t>
+          <t>Q2 draft: 1-day LOT.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>S10. CART_INIT carries through LOT boundary</t>
+          <t>S10. CART_INIT carryover</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>First add medication appears in LOT1, CAR-T occurs within 45 days of that add.</t>
+          <t>CAR-T within 45d of first add in LOT1.</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Per LOT1 spec: LOT1_BASE_END_REASON = CART_INIT and LOT1_BASE_END_DT = FIRST_CART_DT - 1. LOT2_START_TYPE = CART; FIRST_CART_DT = LOT2_START_DT.</t>
+          <t>LOT1 ends with CART_INIT (LOT1 spec). LOT2_START_TYPE=CART.</t>
         </is>
       </c>
     </row>
@@ -4216,13 +4093,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -4261,12 +4138,12 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Should LOT2-5 use the same 90-day discontinuation gap as LOT1?</t>
+          <t>90-day discontinuation gap inherited from LOT1?</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Yes - inherit unless protocol amendment says otherwise.</t>
+          <t>Draft: yes.</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
@@ -4288,12 +4165,12 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Span of an ALLO-only LOT: single day (start=end=ALLO_DT) or extending until next agent?</t>
+          <t>ALLO LOT span: single day or until next agent?</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Draft: single day (consistent with 'ALLO contains no MM therapies'). Aligns with Apr 22 discussion of one-day SCT events.</t>
+          <t>Draft: single day (start=end=ALLO_DT).</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
@@ -4315,12 +4192,12 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Span of a CAR-T LOT when no consolidation agents within 45 days?</t>
+          <t>CAR-T LOT span when no consolidation agents in 45d?</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Draft: LOT spans FIRST_CART_DT to FIRST_CART_DT (1 day) or to last consolidation MAP_END_DT if any agents within 45d.</t>
+          <t>Draft: 1 day, else through last consolidation MAP_END_DT.</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -4342,12 +4219,12 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>If patient receives CAR-T during LOT1 induction window (CART_INIT), where does the next AUTO go?</t>
+          <t>CART_INIT in LOT1 -&gt; LOT2 = CART. Next AUTO -&gt; LOT3 with SCT_AUTO?</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Per LOT1 spec, LOT1 ends day before CAR-T; CAR-T is LOT2. A subsequent AUTO would start LOT3 with SCT_AUTO trigger.</t>
+          <t>Draft: yes.</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -4369,12 +4246,12 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Should LOTN_BASE_END_REASON include MAINTENANCE_END (Rule 8) for LOT2-5?</t>
+          <t>Include MAINTENANCE_END (protocol Rule 8) as LOTN end reason?</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Draft: NO - follows current LOT1 CODE behaviour (no standalone maintenance LOT) rather than the protocol Rule 8 wording. Use contains_mtx_reg_LOTN flag only. If the team later reverses this for LOT1, LOT2-5 should follow.</t>
+          <t>Draft: no - follow current LOT1 code (descriptive flag only).</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -4396,12 +4273,12 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Maximum LOT cap = 5 even if patient continues to switch therapies?</t>
+          <t>Cap LOTs at 5?</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Draft: yes, cap at LOT5 per study scope. Anything after LOT5 collapses into a 'LOT5+' indicator (TBD).</t>
+          <t>Draft: yes; LOT5+ indicator TBD.</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -4423,12 +4300,12 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Should LOTN_TX_AUTO_FLG include AUTOs that occurred during LOT_(N-1) but were attributed to LOT_(N-1)?</t>
+          <t>AUTO flags LOT-scoped to [LOTN_START_DT, LOTN_BASE_END_DT]?</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Draft: NO - AUTO flags are LOT-specific; only AUTOs with FST_DT within [LOTN_START_DT, LOTN_BASE_END_DT].</t>
+          <t>Draft: yes.</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -4450,12 +4327,12 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Steroids leak (LOT1 finding H1) - confirm fix is applied to LOT2-5 induction &amp; first-add candidates.</t>
+          <t>Confirm steroid filter applied (LOT1 H1).</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Yes - all induction filters and first_add_candidates CTEs must include MAP_MED_CLASS != 'STEROID'.</t>
+          <t>Required: MAP_MED_CLASS != 'STEROID' in induction + first-add CTEs.</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -4477,12 +4354,12 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Off-by-one tandem (LOT1 finding H2) - same fix for LOT2-5.</t>
+          <t>Confirm tandem off-by-one fix (LOT1 H2).</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Yes - drop +1 in datediff for tandem window check; window is &gt;=60 AND &lt;=180 days.</t>
+          <t>Required: drop +1 in datediff; window &gt;=60 AND &lt;=180.</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -4504,12 +4381,12 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Output table: should we emit one row per LOT (long format) with LOT_NUM column, or one wide row per patient?</t>
+          <t>Output shape: long (one row per LOT) vs wide?</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Draft: long format (patient_id, LOT_NUM, start, end, reason, regimen) + a wide pivot for analytic convenience.</t>
+          <t>Draft: long primary + wide pivot.</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -4531,12 +4408,12 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>CAR-T consolidation window: 45 vs 30 days.</t>
+          <t>CAR-T consolidation: 45 vs 30 days?</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>RESOLVED: 45 days. Per Apr 22 study-team decision; supersedes the 30-day language in the older protocol extract. Document as Apr 22 decision in spec, NOT 'per protocol'.</t>
+          <t>RESOLVED: 45 days (Apr 22 decision; not 'per protocol').</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -4558,12 +4435,12 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Disenrollment as a LOT end event: primary vs sensitivity treatment.</t>
+          <t>Disenrollment as end event?</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>RESOLVED: PRIMARY analysis ignores disenrollment - LOT N ends only on regimen events, SCT/CAR-T events, death, or study_end. SENSITIVITY analysis (CENSOR_AT_DISENROLLMENT=TRUE) caps observation at ENDDATE_CE = min(YMDOD, ELIGEND, study_end) and emits DISENROLLMENT as the end reason when ELIGEND binds. Spec requires the implementation to label sensitivity reason DISENROLLMENT (not collapse to STUDY_END as current LOT1 code does).</t>
+          <t>RESOLVED: PRIMARY ignores; SENSITIVITY caps via ENDDATE_CE and emits DISENROLLMENT (do NOT collapse to STUDY_END).</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -4574,6 +4451,60 @@
       <c r="E13" s="7" t="inlineStr">
         <is>
           <t>Resolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Flag prefix LOTN_TX_ vs LOTN_SCT_ - LOT1 uses LOT1_SCT_AUTO_*FLG.</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Draft uses LOTN_TX_AUTO_*FLG; consider aligning to LOTN_SCT_AUTO_*FLG.</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Onkar / Julia</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Same-day end-reason priority for LOT2-5 - inherits LOT1?</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Draft: SCT_ALLO &gt; SCT_CART &gt; SCT_AUTO &gt; CART_INIT &gt; MED_ADD &gt; DISCONTINUATION &gt; DEATH &gt; STUDY_END (DISENROLLMENT in sensitivity). Confirm.</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Julia</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -5424,7 +5355,7 @@
     <row r="12" ht="50" customHeight="1">
       <c r="A12" s="43" t="inlineStr">
         <is>
-          <t>Same-day tie-break priority (highest wins): SCT_ALLO &gt; SCT_CART &gt; SCT_AUTO (unplanned) &gt; CART_INIT &gt; MED_ADD &gt; DISCONTINUATION &gt; DEATH &gt; STUDY_END (PRIMARY); DISENROLLMENT slots between DEATH and STUDY_END in SENSITIVITY only.</t>
+          <t>Same-day priority (DRAFT, inherits LOT1 - confirm): SCT_ALLO &gt; SCT_CART &gt; SCT_AUTO &gt; CART_INIT &gt; MED_ADD &gt; DISCONTINUATION &gt; DEATH &gt; STUDY_END. Sensitivity adds DISENROLLMENT before STUDY_END.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LOT2-5 spec: fix decision-flow logic; align ALLO example to Q2 pending
- Decision_Flow rewritten as date-driven: collect candidate trigger
  dates (d_MED, d_ALLO, d_CART, d_AUTO), pick min, then tie-break by
  type only on identical dates. Replaces the type-first ordering that
  could pick a later ALLO/CART over an earlier MED.
- Drop the 'isolated AUTO in a new line' phrasing; AUTO trigger is
  strictly 'first UNPLANNED AUTO >180d after prior AUTO'.
- Worked Example B (ALLO LOT): mark LOTN_BASE_END_DT and
  LOTN_BASE_END_REASON as PENDING Q2 with both candidate values
  (single-day=2025-09-15, SCT_ALLO; extend-to-next=2025-12-09, MED_ADD)
  so they no longer disagree.
</commit_message>
<xml_diff>
--- a/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
+++ b/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
@@ -1188,7 +1188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2287,11 +2287,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="C45" s="9" t="inlineStr">
-        <is>
-          <t>Trigger type is SCT_ALLO.</t>
-        </is>
-      </c>
+      <c r="C45" s="9" t="inlineStr"/>
       <c r="D45" s="9" t="n"/>
       <c r="E45" s="9" t="n"/>
       <c r="F45" s="9" t="n"/>
@@ -2301,17 +2297,17 @@
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>LOTN_BASE_END_DT (draft)</t>
+          <t>LOTN_BASE_END_DT</t>
         </is>
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>2025-09-15</t>
+          <t>PENDING Q2</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Draft Q2 assumption: single-day LOT (start = end = ALLO_DT). Next agent (DARA on 2025-12-10) opens LOT3.</t>
+          <t>Q2 draft (single-day): 2025-09-15. Alternative (extend to next agent): 2025-12-09.</t>
         </is>
       </c>
       <c r="D46" s="9" t="n"/>
@@ -2328,12 +2324,12 @@
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>MED_ADD</t>
+          <t>PENDING Q2</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>DARA on 2025-12-10 is the next event; LOT2 ends the day before LOT3 starts. (Pending Q2.)</t>
+          <t>Q2 draft (single-day): SCT_ALLO. Alternative (extend to next agent): MED_ADD.</t>
         </is>
       </c>
       <c r="D47" s="9" t="n"/>
@@ -2342,83 +2338,83 @@
       <c r="G47" s="9" t="n"/>
       <c r="H47" s="9" t="n"/>
     </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="8" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>LOT3_START_DT</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>DARA - first MM agent after LOT2.</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="n"/>
+      <c r="E48" s="9" t="n"/>
+      <c r="F48" s="9" t="n"/>
+      <c r="G48" s="9" t="n"/>
+      <c r="H48" s="9" t="n"/>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>WORKED EXAMPLE C - LOT2 starts on an unplanned autologous SCT</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="60" customHeight="1">
-      <c r="A51" s="9" t="inlineStr">
+    <row r="52" ht="60" customHeight="1">
+      <c r="A52" s="9" t="inlineStr">
         <is>
           <t>Single AUTO 2025-03-01 in LOT1; second AUTO 2025-10-15 (228d later, unplanned). LOT1 ends 2025-10-14; LOT2 starts on AUTO.</t>
         </is>
       </c>
-      <c r="B51" s="10" t="n"/>
-      <c r="C51" s="10" t="n"/>
-      <c r="D51" s="10" t="n"/>
-      <c r="E51" s="10" t="n"/>
-      <c r="F51" s="10" t="n"/>
-      <c r="G51" s="10" t="n"/>
-      <c r="H51" s="11" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="12" t="inlineStr">
+      <c r="B52" s="10" t="n"/>
+      <c r="C52" s="10" t="n"/>
+      <c r="D52" s="10" t="n"/>
+      <c r="E52" s="10" t="n"/>
+      <c r="F52" s="10" t="n"/>
+      <c r="G52" s="10" t="n"/>
+      <c r="H52" s="11" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="12" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="B52" s="12" t="inlineStr">
+      <c r="B53" s="12" t="inlineStr">
         <is>
           <t>Value for this patient</t>
         </is>
       </c>
-      <c r="C52" s="12" t="inlineStr">
+      <c r="C53" s="12" t="inlineStr">
         <is>
           <t>How it was derived</t>
         </is>
       </c>
-      <c r="D52" s="12" t="n"/>
-      <c r="E52" s="12" t="n"/>
-      <c r="F52" s="12" t="n"/>
-      <c r="G52" s="12" t="n"/>
-      <c r="H52" s="12" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="13" t="inlineStr">
-        <is>
-          <t>LOT_NUM</t>
-        </is>
-      </c>
-      <c r="B53" s="9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C53" s="9" t="inlineStr"/>
-      <c r="D53" s="9" t="n"/>
-      <c r="E53" s="9" t="n"/>
-      <c r="F53" s="9" t="n"/>
-      <c r="G53" s="9" t="n"/>
-      <c r="H53" s="9" t="n"/>
+      <c r="D53" s="12" t="n"/>
+      <c r="E53" s="12" t="n"/>
+      <c r="F53" s="12" t="n"/>
+      <c r="G53" s="12" t="n"/>
+      <c r="H53" s="12" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>LOTN_START_DT</t>
+          <t>LOT_NUM</t>
         </is>
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>2025-10-15</t>
-        </is>
-      </c>
-      <c r="C54" s="9" t="inlineStr">
-        <is>
-          <t>Unplanned AUTO date (&gt;180d after prior AUTO).</t>
-        </is>
-      </c>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr"/>
       <c r="D54" s="9" t="n"/>
       <c r="E54" s="9" t="n"/>
       <c r="F54" s="9" t="n"/>
@@ -2428,17 +2424,17 @@
     <row r="55">
       <c r="A55" s="13" t="inlineStr">
         <is>
-          <t>LOTN_START_TYPE</t>
+          <t>LOTN_START_DT</t>
         </is>
       </c>
       <c r="B55" s="9" t="inlineStr">
         <is>
-          <t>SCT_AUTO</t>
+          <t>2025-10-15</t>
         </is>
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>Unplanned AUTO is a first-class LOT-start trigger. (Planned tandem 60-180d would NOT start a new LOT.)</t>
+          <t>Unplanned AUTO date (&gt;180d after prior AUTO).</t>
         </is>
       </c>
       <c r="D55" s="9" t="n"/>
@@ -2450,17 +2446,17 @@
     <row r="56">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>INDUCTION_WINDOW_DAYS</t>
+          <t>LOTN_START_TYPE</t>
         </is>
       </c>
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>SCT_AUTO</t>
         </is>
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>LOT2 captures any post-AUTO agents within [2025-10-15, 2025-11-13].</t>
+          <t>Unplanned AUTO is a first-class LOT-start trigger. (Planned tandem 60-180d would NOT start a new LOT.)</t>
         </is>
       </c>
       <c r="D56" s="9" t="n"/>
@@ -2472,17 +2468,17 @@
     <row r="57">
       <c r="A57" s="13" t="inlineStr">
         <is>
-          <t>LOTN_TX_AUTO_FLG</t>
+          <t>INDUCTION_WINDOW_DAYS</t>
         </is>
       </c>
       <c r="B57" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>AUTO occurred during LOT2.</t>
+          <t>LOT2 captures any post-AUTO agents within [2025-10-15, 2025-11-13].</t>
         </is>
       </c>
       <c r="D57" s="9" t="n"/>
@@ -2494,7 +2490,7 @@
     <row r="58">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>LOTN_TX_AUTO_SING_FLG</t>
+          <t>LOTN_TX_AUTO_FLG</t>
         </is>
       </c>
       <c r="B58" s="9" t="inlineStr">
@@ -2504,7 +2500,7 @@
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>Single AUTO during LOT2 (no second AUTO within tandem window).</t>
+          <t>AUTO occurred during LOT2.</t>
         </is>
       </c>
       <c r="D58" s="9" t="n"/>
@@ -2516,23 +2512,45 @@
     <row r="59">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>LOTN_TX_AUTO_TAND_FLG</t>
+          <t>LOTN_TX_AUTO_SING_FLG</t>
         </is>
       </c>
       <c r="B59" s="9" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C59" s="9" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>Single AUTO during LOT2 (no second AUTO within tandem window).</t>
+        </is>
+      </c>
       <c r="D59" s="9" t="n"/>
       <c r="E59" s="9" t="n"/>
       <c r="F59" s="9" t="n"/>
       <c r="G59" s="9" t="n"/>
       <c r="H59" s="9" t="n"/>
     </row>
+    <row r="60">
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>LOTN_TX_AUTO_TAND_FLG</t>
+        </is>
+      </c>
+      <c r="B60" s="9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr"/>
+      <c r="D60" s="9" t="n"/>
+      <c r="E60" s="9" t="n"/>
+      <c r="F60" s="9" t="n"/>
+      <c r="G60" s="9" t="n"/>
+      <c r="H60" s="9" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="36">
+  <mergeCells count="37">
     <mergeCell ref="C25:H25"/>
     <mergeCell ref="C41:H41"/>
     <mergeCell ref="C47:H47"/>
@@ -2547,12 +2565,12 @@
     <mergeCell ref="C56:H56"/>
     <mergeCell ref="C59:H59"/>
     <mergeCell ref="C46:H46"/>
+    <mergeCell ref="C60:H60"/>
     <mergeCell ref="C27:H27"/>
-    <mergeCell ref="C52:H52"/>
     <mergeCell ref="C23:H23"/>
     <mergeCell ref="C39:H39"/>
+    <mergeCell ref="C48:H48"/>
     <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A50:H50"/>
     <mergeCell ref="C32:H32"/>
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="C57:H57"/>
@@ -2566,6 +2584,7 @@
     <mergeCell ref="C58:H58"/>
     <mergeCell ref="A20:H20"/>
     <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A52:H52"/>
     <mergeCell ref="C45:H45"/>
     <mergeCell ref="C26:H26"/>
     <mergeCell ref="C29:H29"/>
@@ -5158,7 +5177,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Read top-to-bottom. Each event evaluates AFTER LOT_N_BASE_END_DT. The earliest qualifying trigger determines LOT_(N+1)_START_DT and LOTN+1_START_TYPE.</t>
+          <t>Date-driven, NOT type-driven. Step 1: collect candidate dates. Step 2: pick earliest. Step 3: tie-break by type only if multiple triggers fall on that same date.</t>
         </is>
       </c>
     </row>
@@ -5170,17 +5189,17 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Question</t>
+          <t>Action</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>If YES</t>
+          <t>Detail</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>If NO -&gt; next step</t>
+          <t>Output</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -5197,22 +5216,26 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Is there an ALLO SCT after LOT_N ended?</t>
+          <t>Collect candidate trigger dates AFTER LOT_N_BASE_END_DT.</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>LOT_(N+1) starts at ALLO_DT. LOTN+1_START_TYPE = SCT_ALLO. ALLO LOT contains NO MM therapies.</t>
+          <t>Compute, for each trigger type, the earliest qualifying date (if any):
+  d_MED   = first non-steroid MM agent MAP_START_DT (excl. permissible biosimilar subs)
+  d_ALLO  = first ALLO SCT date
+  d_CART  = first CAR-T infusion date (FIRST_CART_DT)
+  d_AUTO  = first UNPLANNED AUTO date (&gt;180d after prior AUTO in LOT_N).</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Step 2</t>
+          <t>Up to 4 candidate dates</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>ALLO always wins ties on the same day.</t>
+          <t>Planned/single/tandem AUTO (60-180d intervals) is a CONTINUATION and is NOT a candidate.</t>
         </is>
       </c>
     </row>
@@ -5224,22 +5247,22 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Is there a CAR-T infusion after LOT_N ended?</t>
+          <t>Pick the earliest candidate date.</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>LOT_(N+1) starts at FIRST_CART_DT. LOTN+1_START_TYPE = CART. Agents within 45d are consolidated (Apr 22 decision).</t>
+          <t>LOT_(N+1)_START_DT = min(d_MED, d_ALLO, d_CART, d_AUTO).</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Step 3</t>
+          <t>LOT_(N+1)_START_DT</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>CAR-T outranks AUTO and MED on tie.</t>
+          <t>An earlier MED beats a later ALLO/CART/AUTO.</t>
         </is>
       </c>
     </row>
@@ -5251,104 +5274,99 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Is there an UNPLANNED AUTO SCT after LOT_N ended?
-(&gt;180d after the prior AUTO in LOT_N, OR an isolated AUTO in a new line)</t>
+          <t>If exactly one candidate equals that earliest date, set its type.</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>LOT_(N+1) starts at AUTO_DT. LOTN+1_START_TYPE = SCT_AUTO.</t>
+          <t>LOTN+1_START_TYPE = the type of the unique earliest candidate.</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Step 4</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>Planned/single/tandem AUTO within 60-180d of a prior AUTO is a CONTINUATION - it does NOT start a new LOT.</t>
-        </is>
-      </c>
+          <t>LOTN+1_START_TYPE</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr"/>
     </row>
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3a</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Is there a new MM oncology agent (non-steroid, non-permissible-substitute) after LOT_N ended?</t>
+          <t>Same-day tie-break (DRAFT, inherits LOT1 - confirm).</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>LOT_(N+1) starts at MAP_START_DT of that agent. LOTN+1_START_TYPE = MED.</t>
+          <t>If multiple triggers share LOT_(N+1)_START_DT: SCT_ALLO &gt; CART &gt; SCT_AUTO &gt; MED.</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Step 5</t>
+          <t>LOTN+1_START_TYPE</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Steroids alone do NOT start a LOT. Biosimilar substitutions do NOT start a LOT.</t>
+          <t>Tie-breaks ONLY on identical dates - never overrides date order.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Has DEATH (YMDOD) or STUDY_END been reached?</t>
+          <t>If no candidate dates exist, evaluate end-of-follow-up.</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Follow-up ends. No LOT_(N+1).</t>
+          <t>If DEATH (YMDOD) or STUDY_END is reached, no LOT_(N+1).</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Step 6 (sensitivity)</t>
+          <t>No LOT_(N+1)</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>PRIMARY analysis closes here.</t>
+          <t>PRIMARY analysis closes here. Disenrollment is NOT a primary closure.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5 (SENSITIVITY)</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>SENSITIVITY ONLY: is CENSOR_AT_DISENROLLMENT = TRUE and ELIGEND earliest?</t>
+          <t>If CENSOR_AT_DISENROLLMENT = TRUE, additionally cap observation at ELIGEND.</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Sensitivity output caps at ENDDATE_CE; LOTN_BASE_END_REASON_CE_SENS = DISENROLLMENT.</t>
+          <t>LOTN_BASE_END_DT_CE_SENS = min(LOTN_BASE_END_DT, ELIGEND); reason = DISENROLLMENT when ELIGEND binds.</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>End</t>
+          <t>Sensitivity outputs only</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Primary analysis ignores ELIGEND. See Q12.</t>
+          <t>Does not affect LOT_(N+1) start. See Q12.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LOT2-5 spec: fix Example A maintenance flag; tighten d_AUTO; relabel decision-flow footer
- Worked Example A: contains_mtx_reg_LOTN was incorrectly set to 1.
  DARA + LENA regimen has BOTH agents on the mono-maintenance list, so
  there is no non-maintenance anchor. Corrected to 0 with the right
  rationale. Also dropped the redundant constants from the patient
  values column (INDUCTION_WINDOW_DAYS).
- Decision_Flow d_AUTO: comparison is to the most recent prior AUTO in
  the patient's history (not strictly LOT_N). If no prior AUTO at all,
  AUTO is not a LOT-start candidate.
- Decision_Flow footer: explicitly labelled END-REASON priority and
  cross-referenced to LOTN_BASE_END_REASON in tab 4, so reviewers can
  not confuse it with the LOT-start tie-break in Step 3a (P3 fix).
</commit_message>
<xml_diff>
--- a/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
+++ b/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
@@ -1188,7 +1188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1882,11 +1882,7 @@
           <t>2</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>Sequential index after LOT1.</t>
-        </is>
-      </c>
+      <c r="C23" s="9" t="inlineStr"/>
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="9" t="n"/>
       <c r="F23" s="9" t="n"/>
@@ -1906,7 +1902,7 @@
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Earliest competing trigger after LOT1_BASE_END_DT (2025-08-19) is the new MM agent DARA on 2025-08-20.</t>
+          <t>Earliest trigger after LOT1_BASE_END_DT (2025-08-19) = DARA.</t>
         </is>
       </c>
       <c r="D24" s="9" t="n"/>
@@ -1926,11 +1922,7 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>Trigger was a new medication (no SCT/CAR-T present).</t>
-        </is>
-      </c>
+      <c r="C25" s="9" t="inlineStr"/>
       <c r="D25" s="9" t="n"/>
       <c r="E25" s="9" t="n"/>
       <c r="F25" s="9" t="n"/>
@@ -1940,17 +1932,17 @@
     <row r="26">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>INDUCTION_WINDOW_DAYS</t>
+          <t>LOTN_BASE_MEDS</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>DARA, LENA</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>LOT2 uses the 30-day induction window (vs 60 for LOT1).</t>
+          <t>Window [2025-08-20, 2025-09-18]. DEXA excluded (steroid).</t>
         </is>
       </c>
       <c r="D26" s="9" t="n"/>
@@ -1962,19 +1954,15 @@
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
-          <t>LOTN_BASE_MEDS</t>
+          <t>LOTN_MED_CNT</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>DARA, LENA</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>Within [2025-08-20, 2025-09-18]: DARA (start) and LENA refills. DEXA excluded (steroid).</t>
-        </is>
-      </c>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr"/>
       <c r="D27" s="9" t="n"/>
       <c r="E27" s="9" t="n"/>
       <c r="F27" s="9" t="n"/>
@@ -1984,19 +1972,15 @@
     <row r="28">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>LOTN_MED_CNT</t>
+          <t>LOTN_MED_DARA</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>Two distinct non-steroid agents.</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr"/>
       <c r="D28" s="9" t="n"/>
       <c r="E28" s="9" t="n"/>
       <c r="F28" s="9" t="n"/>
@@ -2006,7 +1990,7 @@
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>LOTN_MED_DARA</t>
+          <t>LOTN_MED_LENA</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
@@ -2014,11 +1998,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>DARA present in LOTN_BASE_MEDS.</t>
-        </is>
-      </c>
+      <c r="C29" s="9" t="inlineStr"/>
       <c r="D29" s="9" t="n"/>
       <c r="E29" s="9" t="n"/>
       <c r="F29" s="9" t="n"/>
@@ -2028,7 +2008,7 @@
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>LOTN_MED_LENA</t>
+          <t>LOTN_CLASS_ANTICD38</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
@@ -2038,7 +2018,7 @@
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>LENA present in LOTN_BASE_MEDS.</t>
+          <t>DARA.</t>
         </is>
       </c>
       <c r="D30" s="9" t="n"/>
@@ -2050,7 +2030,7 @@
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>LOTN_CLASS_ANTICD38</t>
+          <t>LOTN_CLASS_IMMUNOMOD</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
@@ -2060,7 +2040,7 @@
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>DARA is class ANTICD38.</t>
+          <t>LENA.</t>
         </is>
       </c>
       <c r="D31" s="9" t="n"/>
@@ -2072,17 +2052,17 @@
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>LOTN_CLASS_IMMUNOMOD</t>
+          <t>contains_mtx_reg_LOTN</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>LENA is class IMMUNOMOD.</t>
+          <t>BOTH DARA and LENA are valid mono-maintenance agents - no non-maintenance anchor.</t>
         </is>
       </c>
       <c r="D32" s="9" t="n"/>
@@ -2094,102 +2074,98 @@
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>contains_mtx_reg_LOTN</t>
+          <t>LOTN_ALLO_LOT_FLG / LOTN_CART_LOT_FLG</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>LENA is a valid mono-maintenance agent (a); DARA is the non-maintenance anchor (b).</t>
-        </is>
-      </c>
+          <t>0 / 0</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr"/>
       <c r="D33" s="9" t="n"/>
       <c r="E33" s="9" t="n"/>
       <c r="F33" s="9" t="n"/>
       <c r="G33" s="9" t="n"/>
       <c r="H33" s="9" t="n"/>
     </row>
-    <row r="34">
-      <c r="A34" s="13" t="inlineStr">
-        <is>
-          <t>LOTN_ALLO_LOT_FLG / LOTN_CART_LOT_FLG</t>
-        </is>
-      </c>
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t>0 / 0</t>
-        </is>
-      </c>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t>No ALLO or CAR-T trigger.</t>
-        </is>
-      </c>
-      <c r="D34" s="9" t="n"/>
-      <c r="E34" s="9" t="n"/>
-      <c r="F34" s="9" t="n"/>
-      <c r="G34" s="9" t="n"/>
-      <c r="H34" s="9" t="n"/>
-    </row>
-    <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="8" t="inlineStr">
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>WORKED EXAMPLE B - LOT2 starts on an allogeneic SCT</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="60" customHeight="1">
-      <c r="A38" s="9" t="inlineStr">
+    <row r="37" ht="60" customHeight="1">
+      <c r="A37" s="9" t="inlineStr">
         <is>
           <t>VRd in LOT1; ALLO on 2025-09-15 (LOT1 ends 2025-09-14). Next MM therapy DARA on 2025-12-10 starts LOT3.</t>
         </is>
       </c>
-      <c r="B38" s="10" t="n"/>
-      <c r="C38" s="10" t="n"/>
-      <c r="D38" s="10" t="n"/>
-      <c r="E38" s="10" t="n"/>
-      <c r="F38" s="10" t="n"/>
-      <c r="G38" s="10" t="n"/>
-      <c r="H38" s="11" t="n"/>
+      <c r="B37" s="10" t="n"/>
+      <c r="C37" s="10" t="n"/>
+      <c r="D37" s="10" t="n"/>
+      <c r="E37" s="10" t="n"/>
+      <c r="F37" s="10" t="n"/>
+      <c r="G37" s="10" t="n"/>
+      <c r="H37" s="11" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>Value for this patient</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>How it was derived</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="n"/>
+      <c r="E38" s="12" t="n"/>
+      <c r="F38" s="12" t="n"/>
+      <c r="G38" s="12" t="n"/>
+      <c r="H38" s="12" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="12" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
-      </c>
-      <c r="B39" s="12" t="inlineStr">
-        <is>
-          <t>Value for this patient</t>
-        </is>
-      </c>
-      <c r="C39" s="12" t="inlineStr">
-        <is>
-          <t>How it was derived</t>
-        </is>
-      </c>
-      <c r="D39" s="12" t="n"/>
-      <c r="E39" s="12" t="n"/>
-      <c r="F39" s="12" t="n"/>
-      <c r="G39" s="12" t="n"/>
-      <c r="H39" s="12" t="n"/>
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>LOT_NUM</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr"/>
+      <c r="D39" s="9" t="n"/>
+      <c r="E39" s="9" t="n"/>
+      <c r="F39" s="9" t="n"/>
+      <c r="G39" s="9" t="n"/>
+      <c r="H39" s="9" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>LOT_NUM</t>
+          <t>LOTN_START_DT</t>
         </is>
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C40" s="9" t="inlineStr"/>
+          <t>2025-09-15</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>ALLO_DT (always starts a new LOT).</t>
+        </is>
+      </c>
       <c r="D40" s="9" t="n"/>
       <c r="E40" s="9" t="n"/>
       <c r="F40" s="9" t="n"/>
@@ -2199,19 +2175,15 @@
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>LOTN_START_DT</t>
+          <t>LOTN_START_TYPE</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>2025-09-15</t>
-        </is>
-      </c>
-      <c r="C41" s="9" t="inlineStr">
-        <is>
-          <t>ALLO_DT (always starts a new LOT).</t>
-        </is>
-      </c>
+          <t>SCT_ALLO</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr"/>
       <c r="D41" s="9" t="n"/>
       <c r="E41" s="9" t="n"/>
       <c r="F41" s="9" t="n"/>
@@ -2221,15 +2193,19 @@
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>LOTN_START_TYPE</t>
+          <t>LOTN_BASE_MEDS</t>
         </is>
       </c>
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>SCT_ALLO</t>
-        </is>
-      </c>
-      <c r="C42" s="9" t="inlineStr"/>
+          <t>(empty)</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>ALLO LOT contains NO MM therapies.</t>
+        </is>
+      </c>
       <c r="D42" s="9" t="n"/>
       <c r="E42" s="9" t="n"/>
       <c r="F42" s="9" t="n"/>
@@ -2239,19 +2215,15 @@
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>LOTN_BASE_MEDS</t>
+          <t>LOTN_MED_CNT</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>(empty)</t>
-        </is>
-      </c>
-      <c r="C43" s="9" t="inlineStr">
-        <is>
-          <t>ALLO LOT contains NO MM therapies.</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr"/>
       <c r="D43" s="9" t="n"/>
       <c r="E43" s="9" t="n"/>
       <c r="F43" s="9" t="n"/>
@@ -2261,12 +2233,12 @@
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>LOTN_MED_CNT</t>
+          <t>LOTN_ALLO_LOT_FLG</t>
         </is>
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr"/>
@@ -2279,15 +2251,19 @@
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>LOTN_ALLO_LOT_FLG</t>
+          <t>LOTN_BASE_END_DT</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C45" s="9" t="inlineStr"/>
+          <t>PENDING Q2</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Q2 draft (single-day): 2025-09-15. Alternative (extend to next agent): 2025-12-09.</t>
+        </is>
+      </c>
       <c r="D45" s="9" t="n"/>
       <c r="E45" s="9" t="n"/>
       <c r="F45" s="9" t="n"/>
@@ -2297,7 +2273,7 @@
     <row r="46">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>LOTN_BASE_END_DT</t>
+          <t>LOTN_BASE_END_REASON</t>
         </is>
       </c>
       <c r="B46" s="9" t="inlineStr">
@@ -2307,7 +2283,7 @@
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Q2 draft (single-day): 2025-09-15. Alternative (extend to next agent): 2025-12-09.</t>
+          <t>Q2 draft (single-day): SCT_ALLO. Alternative (extend to next agent): MED_ADD.</t>
         </is>
       </c>
       <c r="D46" s="9" t="n"/>
@@ -2319,17 +2295,17 @@
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>LOTN_BASE_END_REASON</t>
+          <t>LOT3_START_DT</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>PENDING Q2</t>
+          <t>2025-12-10</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>Q2 draft (single-day): SCT_ALLO. Alternative (extend to next agent): MED_ADD.</t>
+          <t>DARA - first MM agent after LOT2.</t>
         </is>
       </c>
       <c r="D47" s="9" t="n"/>
@@ -2338,83 +2314,83 @@
       <c r="G47" s="9" t="n"/>
       <c r="H47" s="9" t="n"/>
     </row>
-    <row r="48">
-      <c r="A48" s="13" t="inlineStr">
-        <is>
-          <t>LOT3_START_DT</t>
-        </is>
-      </c>
-      <c r="B48" s="9" t="inlineStr">
-        <is>
-          <t>2025-12-10</t>
-        </is>
-      </c>
-      <c r="C48" s="9" t="inlineStr">
-        <is>
-          <t>DARA - first MM agent after LOT2.</t>
-        </is>
-      </c>
-      <c r="D48" s="9" t="n"/>
-      <c r="E48" s="9" t="n"/>
-      <c r="F48" s="9" t="n"/>
-      <c r="G48" s="9" t="n"/>
-      <c r="H48" s="9" t="n"/>
-    </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="8" t="inlineStr">
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>WORKED EXAMPLE C - LOT2 starts on an unplanned autologous SCT</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="60" customHeight="1">
-      <c r="A52" s="9" t="inlineStr">
+    <row r="51" ht="60" customHeight="1">
+      <c r="A51" s="9" t="inlineStr">
         <is>
           <t>Single AUTO 2025-03-01 in LOT1; second AUTO 2025-10-15 (228d later, unplanned). LOT1 ends 2025-10-14; LOT2 starts on AUTO.</t>
         </is>
       </c>
-      <c r="B52" s="10" t="n"/>
-      <c r="C52" s="10" t="n"/>
-      <c r="D52" s="10" t="n"/>
-      <c r="E52" s="10" t="n"/>
-      <c r="F52" s="10" t="n"/>
-      <c r="G52" s="10" t="n"/>
-      <c r="H52" s="11" t="n"/>
+      <c r="B51" s="10" t="n"/>
+      <c r="C51" s="10" t="n"/>
+      <c r="D51" s="10" t="n"/>
+      <c r="E51" s="10" t="n"/>
+      <c r="F51" s="10" t="n"/>
+      <c r="G51" s="10" t="n"/>
+      <c r="H51" s="11" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="12" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>Value for this patient</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="inlineStr">
+        <is>
+          <t>How it was derived</t>
+        </is>
+      </c>
+      <c r="D52" s="12" t="n"/>
+      <c r="E52" s="12" t="n"/>
+      <c r="F52" s="12" t="n"/>
+      <c r="G52" s="12" t="n"/>
+      <c r="H52" s="12" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="12" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
-      </c>
-      <c r="B53" s="12" t="inlineStr">
-        <is>
-          <t>Value for this patient</t>
-        </is>
-      </c>
-      <c r="C53" s="12" t="inlineStr">
-        <is>
-          <t>How it was derived</t>
-        </is>
-      </c>
-      <c r="D53" s="12" t="n"/>
-      <c r="E53" s="12" t="n"/>
-      <c r="F53" s="12" t="n"/>
-      <c r="G53" s="12" t="n"/>
-      <c r="H53" s="12" t="n"/>
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>LOT_NUM</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr"/>
+      <c r="D53" s="9" t="n"/>
+      <c r="E53" s="9" t="n"/>
+      <c r="F53" s="9" t="n"/>
+      <c r="G53" s="9" t="n"/>
+      <c r="H53" s="9" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>LOT_NUM</t>
+          <t>LOTN_START_DT</t>
         </is>
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C54" s="9" t="inlineStr"/>
+          <t>2025-10-15</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>Unplanned AUTO date (&gt;180d after prior AUTO).</t>
+        </is>
+      </c>
       <c r="D54" s="9" t="n"/>
       <c r="E54" s="9" t="n"/>
       <c r="F54" s="9" t="n"/>
@@ -2424,17 +2400,17 @@
     <row r="55">
       <c r="A55" s="13" t="inlineStr">
         <is>
-          <t>LOTN_START_DT</t>
+          <t>LOTN_START_TYPE</t>
         </is>
       </c>
       <c r="B55" s="9" t="inlineStr">
         <is>
-          <t>2025-10-15</t>
+          <t>SCT_AUTO</t>
         </is>
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>Unplanned AUTO date (&gt;180d after prior AUTO).</t>
+          <t>Unplanned AUTO is a first-class LOT-start trigger. (Planned tandem 60-180d would NOT start a new LOT.)</t>
         </is>
       </c>
       <c r="D55" s="9" t="n"/>
@@ -2446,17 +2422,17 @@
     <row r="56">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>LOTN_START_TYPE</t>
+          <t>INDUCTION_WINDOW_DAYS</t>
         </is>
       </c>
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>SCT_AUTO</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>Unplanned AUTO is a first-class LOT-start trigger. (Planned tandem 60-180d would NOT start a new LOT.)</t>
+          <t>LOT2 captures any post-AUTO agents within [2025-10-15, 2025-11-13].</t>
         </is>
       </c>
       <c r="D56" s="9" t="n"/>
@@ -2468,17 +2444,17 @@
     <row r="57">
       <c r="A57" s="13" t="inlineStr">
         <is>
-          <t>INDUCTION_WINDOW_DAYS</t>
+          <t>LOTN_TX_AUTO_FLG</t>
         </is>
       </c>
       <c r="B57" s="9" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>LOT2 captures any post-AUTO agents within [2025-10-15, 2025-11-13].</t>
+          <t>AUTO occurred during LOT2.</t>
         </is>
       </c>
       <c r="D57" s="9" t="n"/>
@@ -2490,7 +2466,7 @@
     <row r="58">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>LOTN_TX_AUTO_FLG</t>
+          <t>LOTN_TX_AUTO_SING_FLG</t>
         </is>
       </c>
       <c r="B58" s="9" t="inlineStr">
@@ -2500,7 +2476,7 @@
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>AUTO occurred during LOT2.</t>
+          <t>Single AUTO during LOT2 (no second AUTO within tandem window).</t>
         </is>
       </c>
       <c r="D58" s="9" t="n"/>
@@ -2512,45 +2488,23 @@
     <row r="59">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>LOTN_TX_AUTO_SING_FLG</t>
+          <t>LOTN_TX_AUTO_TAND_FLG</t>
         </is>
       </c>
       <c r="B59" s="9" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C59" s="9" t="inlineStr">
-        <is>
-          <t>Single AUTO during LOT2 (no second AUTO within tandem window).</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr"/>
       <c r="D59" s="9" t="n"/>
       <c r="E59" s="9" t="n"/>
       <c r="F59" s="9" t="n"/>
       <c r="G59" s="9" t="n"/>
       <c r="H59" s="9" t="n"/>
     </row>
-    <row r="60">
-      <c r="A60" s="13" t="inlineStr">
-        <is>
-          <t>LOTN_TX_AUTO_TAND_FLG</t>
-        </is>
-      </c>
-      <c r="B60" s="9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="C60" s="9" t="inlineStr"/>
-      <c r="D60" s="9" t="n"/>
-      <c r="E60" s="9" t="n"/>
-      <c r="F60" s="9" t="n"/>
-      <c r="G60" s="9" t="n"/>
-      <c r="H60" s="9" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="37">
+  <mergeCells count="36">
     <mergeCell ref="C25:H25"/>
     <mergeCell ref="C41:H41"/>
     <mergeCell ref="C47:H47"/>
@@ -2561,30 +2515,29 @@
     <mergeCell ref="C40:H40"/>
     <mergeCell ref="A51:H51"/>
     <mergeCell ref="C31:H31"/>
+    <mergeCell ref="A36:H36"/>
     <mergeCell ref="C43:H43"/>
     <mergeCell ref="C56:H56"/>
     <mergeCell ref="C59:H59"/>
     <mergeCell ref="C46:H46"/>
-    <mergeCell ref="C60:H60"/>
     <mergeCell ref="C27:H27"/>
+    <mergeCell ref="C52:H52"/>
     <mergeCell ref="C23:H23"/>
     <mergeCell ref="C39:H39"/>
-    <mergeCell ref="C48:H48"/>
     <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A50:H50"/>
     <mergeCell ref="C32:H32"/>
+    <mergeCell ref="C38:H38"/>
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="C57:H57"/>
     <mergeCell ref="C28:H28"/>
     <mergeCell ref="C53:H53"/>
-    <mergeCell ref="C34:H34"/>
     <mergeCell ref="C30:H30"/>
     <mergeCell ref="C33:H33"/>
     <mergeCell ref="C24:H24"/>
     <mergeCell ref="C42:H42"/>
     <mergeCell ref="C58:H58"/>
     <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A52:H52"/>
     <mergeCell ref="C45:H45"/>
     <mergeCell ref="C26:H26"/>
     <mergeCell ref="C29:H29"/>
@@ -5225,7 +5178,7 @@
   d_MED   = first non-steroid MM agent MAP_START_DT (excl. permissible biosimilar subs)
   d_ALLO  = first ALLO SCT date
   d_CART  = first CAR-T infusion date (FIRST_CART_DT)
-  d_AUTO  = first UNPLANNED AUTO date (&gt;180d after prior AUTO in LOT_N).</t>
+  d_AUTO  = first UNPLANNED AUTO date (&gt;180d after the most recent prior AUTO in the patient's history; if no prior AUTO, AUTO is NOT a candidate).</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -5373,7 +5326,7 @@
     <row r="12" ht="50" customHeight="1">
       <c r="A12" s="43" t="inlineStr">
         <is>
-          <t>Same-day priority (DRAFT, inherits LOT1 - confirm): SCT_ALLO &gt; SCT_CART &gt; SCT_AUTO &gt; CART_INIT &gt; MED_ADD &gt; DISCONTINUATION &gt; DEATH &gt; STUDY_END. Sensitivity adds DISENROLLMENT before STUDY_END.</t>
+          <t>END-REASON same-day priority (separate from LOT-start tie-break in Step 3a; DRAFT, inherits LOT1 - confirm): SCT_ALLO &gt; SCT_CART &gt; SCT_AUTO &gt; CART_INIT &gt; MED_ADD &gt; DISCONTINUATION &gt; DEATH &gt; STUDY_END. SENSITIVITY adds DISENROLLMENT before STUDY_END. See LOTN_BASE_END_REASON in tab 4.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LOT2-5 spec: fix accidental formula cells; guard against future regressions
- Three definition cells in 3.LOT2_5_BASE (E15:E17, the contains_mtx_reg
  / ALLO_LOT_FLG / CART_LOT_FLG rows) started with '= 1 when ...' which
  openpyxl stored as Excel formulas. Reworded to 'Flag is 1 when ...'.
- Add _safe() guard in the row writer that raises at build time if any
  cell value starts with =, +, -, or @ (Excel formula triggers), so this
  class of bug surfaces during regeneration rather than as a corrupt
  cell in the workbook.
- Verified the regenerated workbook has 0 formula cells.
</commit_message>
<xml_diff>
--- a/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
+++ b/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
@@ -1742,9 +1742,10 @@
           <t>0/1</t>
         </is>
       </c>
-      <c r="E15" s="7">
-        <f> 1 when LOT N induction has BOTH (a) &gt;=1 valid mono-maintenance agent OR a valid dual combo, AND (b) a non-maintenance anchor. Mono: LENA, BORT, DARA, IXAZ, THAL. Dual: BORT+LENA, CARF+LENA, DARA+LENA.</f>
-        <v/>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Flag is 1 when LOT N induction has BOTH (a) &gt;=1 valid mono-maintenance agent OR a valid dual combo, AND (b) a non-maintenance anchor. Mono: LENA, BORT, DARA, IXAZ, THAL. Dual: BORT+LENA, CARF+LENA, DARA+LENA.</t>
+        </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
@@ -1779,9 +1780,10 @@
           <t>0/1</t>
         </is>
       </c>
-      <c r="E16" s="7">
-        <f> 1 when LOTN_START_TYPE = SCT_ALLO. ALLO LOT contains no MM therapies. Span: see Q2 (draft = single day).</f>
-        <v/>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Flag is 1 when LOTN_START_TYPE = SCT_ALLO. ALLO LOT contains no MM therapies. Span: see Q2 (draft = single day).</t>
+        </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
@@ -1812,9 +1814,10 @@
           <t>0/1</t>
         </is>
       </c>
-      <c r="E17" s="7">
-        <f> 1 when LOTN_START_TYPE = CART. Agents within 45d of FIRST_CART_DT are consolidated into LOT N (Apr 22 decision; see Q11).</f>
-        <v/>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Flag is 1 when LOTN_START_TYPE = CART. Agents within 45d of FIRST_CART_DT are consolidated into LOT N (Apr 22 decision; see Q11).</t>
+        </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Spec: add Q15 - CAR-T LOT end reason (SCT_CART vs DISCONTINUATION)
Surfaces the methodology question raised in code review of the LOT 2-5
builder: when a CAR-T-started LOT has consolidation meds and ends at
the last consolidation MAP_END_DT, the current implementation labels
the reason DISCONTINUATION (it is a runout date). The alternative is
to force SCT_CART for any CAR-T-started LOT regardless of how the
consolidation regimen ends. Defaulted to DISCONTINUATION pending Julia.
</commit_message>
<xml_diff>
--- a/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
+++ b/Apr 18 2026/Program Spec and Scenarios/lot2to5_spec_DRAFT_apr30.xlsx
@@ -4068,7 +4068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4478,6 +4478,33 @@
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>CAR-T LOT end reason when consolidation meds run out: SCT_CART or DISCONTINUATION?</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Draft (current code): DISCONTINUATION - CAR-T LOT spans through last consolidation MAP_END_DT and routes by runout. Alternative: force SCT_CART for any CAR-T-started LOT regardless of how the consolidation regimen ends.</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Julia</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>Open</t>
         </is>

</xml_diff>